<commit_message>
JEST 1.a: role, full acik sinyalini ureten eleman olarak tanimlandi
Role tetikleme hattinda degil: TENU on kanat tam acik cikisina baglanir ve
role kontaginin cikisi MUX B-A (31) girisine kapi full acik sinyali olarak
verilir. Arac tarafinda boyle bir sinyal bulunmadigi icin bu zincir
kurulmustur. Kapi full acikken MUX C-C (16) trigger ucuna 12V gonderir;
kapi tam acik konumdan ciktigi an sinyal duser ve trigger 0V olur, fotosel
12 beamden 2 beame iner.

Role ile ilgili acik nokta kapatildi; KTP MADDE 2 ve 3 role kontagini ve
B-A (31) girisini de olcecek sekilde guncellendi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1jP1JN4GEcVEbhfkZatnJ
</commit_message>
<xml_diff>
--- a/JEST_SOFTWARE_KTP_Guncel.xlsx
+++ b/JEST_SOFTWARE_KTP_Guncel.xlsx
@@ -687,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -777,16 +777,17 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Fotosel, tetikleme (IN) girişinin seviyesine göre iki farklı algılama alanında çalışır: giriş 12V seviyesindeyken geniş algılama alanı (12 beam), düşük seviyedeyken dar algılama alanı (2 beam) devrededir. Bu giriş araç yazılımının çıkışı ile sürülür. Kapı açıkken trigger ucuna 12V verilir ve geniş algılama alanı devrededir; kapı butonuna basılıp kapı kapanmaya başladığı an 12V kesilir ve dar algılama alanına geçilir. Böylece kapı ağzına giren kanatlar algılama alanını tetiklemez, kapı ağzının ortasında duran yolcu ise görülmeye devam eder.</t>
+          <t>Fotosel, tetikleme (IN) girişinin seviyesine göre iki farklı algılama alanında çalışır: kapı tam açık olduğu durumda trigger ucuna 12V verilir ve fotosel 12 beamlik geniş alanda çalışır. Kapı tam açık sinyali araç tarafında hâli hazırda bulunmadığından, TENU üzerindeki ön kanat tam açık sinyalinden bir röle bağlantısı kurulur ve rölenin çıkışı araç yazılımına kapı full açık sinyali olarak verilir. Kapı full açık olduğu durumda araç yazılımı fotoselin trigger ucuna 12V gönderir; kapı tam açık konumundan çıktığı anda 12V kesilir ve 0V verilir. 12V kesildiği anda fotosel 12 beamden 2 beame düşer. Böylece kapı ağzına giren kanatlar algılama alanını tetiklemez, kapı ağzının ortasında duran yolcu ise görülmeye devam eder.</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>1. MUX C-C (16) → fotosel trigger ucuna 12V kapı açık sinyali veren çıkış
-2. Kapı açık → çıkış aktif, trigger ucunda 12V → 12 beam (geniş algılama alanı).
-3. Kapı butonuna basılıp kapı kapanmaya başladığı an → çıkış pasife alınır, 12V kesilir → 2 beam (dar algılama alanı).
-4. Kapı kapalı konumdayken ve kapı açılırken çıkış pasif tutulur.
-5. Tetikleme için röle kullanılmaz; çıkış doğrudan fotosel trigger ucunu sürer.</t>
+          <t>1. MUX B-A (31) ← kapı full açık sinyali (TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır)
+2. MUX C-C (16) → fotosel trigger ucuna 12V kapı açık sinyali veren çıkış
+3. Kapı full açık → çıkış aktif, trigger ucunda 12V → 12 beam (geniş algılama alanı).
+4. Kapı tam açık konumundan çıktığı an → full açık sinyali düşer, çıkış pasife alınır, trigger ucu 0V → 2 beam (dar algılama alanı).
+5. Kapı kapalı konumdayken ve kapı açılırken çıkış pasif tutulur; kapı tam açık konuma ulaştığında yeniden aktif edilir.
+6. Röle bobini TENU ön kanat tam açık çıkışına bağlanır; röle kontağının çıkışı MUX B-A (31) girişine verilir.</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -956,7 +957,7 @@
         <is>
           <t>1. Cluster, araç yazılımına 10 saniye olarak setleme bilgisi gönderir.
 2. Ekranda Telltale 1 aktif edilir.
-3. Sayaç başlangıcı: MUX B-A (31) ← araçtan aldığımız kapı full açık sinyali
+3. Sayaç başlangıcı: MUX B-A (31) ← kapı full açık sinyali (TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır)
 4. Sayaç reset: MUX C-A (12) ← fotoselin engel algılayıp algılamadığının muxa giden pini (Fotosel Output) aktif olduğunda.</t>
         </is>
       </c>
@@ -986,7 +987,7 @@
         <is>
           <t>1. Cluster, araç yazılımına 14 saniye olarak setleme bilgisi gönderir.
 2. Ekranda Telltale 2 aktif edilir.
-3. Sayaç başlangıcı: MUX B-A (31) ← araçtan aldığımız kapı full açık sinyali
+3. Sayaç başlangıcı: MUX B-A (31) ← kapı full açık sinyali (TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır)
 4. Sayaç reset: MUX C-A (12) ← fotoselin engel algılayıp algılamadığının muxa giden pini (Fotosel Output) aktif olduğunda.</t>
         </is>
       </c>
@@ -1016,7 +1017,7 @@
         <is>
           <t>1. Cluster, araç yazılımına 3 saniye olarak setleme bilgisi gönderir.
 2. Ekranda Telltale 3 aktif edilir.
-3. Sayaç başlangıcı: MUX B-A (31) ← araçtan aldığımız kapı full açık sinyali
+3. Sayaç başlangıcı: MUX B-A (31) ← kapı full açık sinyali (TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır)
 4. Sayaç reset: MUX C-A (12) ← fotoselin engel algılayıp algılamadığının muxa giden pini (Fotosel Output) aktif olduğunda.</t>
         </is>
       </c>
@@ -1202,21 +1203,13 @@
     <row r="23" ht="42" customHeight="1">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>3) Blok şemada TENU A5 hattına paralel bağlanan röle görünmektedir. Tetikleme artık MUX C-C (16) çıkışından yapıldığına göre bu rölenin devrede kalıp kalmadığı, kalıyorsa hangi işlevi gördüğü netleştirilmelidir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="42" customHeight="1">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t>4) Fotosel çıkış seviyesi 12V'tur. MUX C-A (12) girişinin bu seviyeyi dijital giriş olarak doğru okuduğu araç üzerinde doğrulanmalıdır.</t>
+          <t>3) Fotosel çıkış seviyesi 12V'tur. MUX C-A (12) girişinin bu seviyeyi dijital giriş olarak doğru okuduğu araç üzerinde doğrulanmalıdır.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A24:E24"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A22:E22"/>
@@ -1390,7 +1383,7 @@
       <c r="C6" s="18" t="n"/>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Kapı tam açık konuma getirilir; MUX C-C (16) çıkışı, fotosel trigger ucu ve MUX B-A (31) girişi ölçülür.</t>
+          <t>Kapı tam açık konuma getirilir; TENU ön kanat tam açık çıkışı, röle kontağı, MUX B-A (31) girişi, MUX C-C (16) çıkışı ve fotosel trigger ucu birlikte ölçülür.</t>
         </is>
       </c>
       <c r="E6" s="18" t="n"/>
@@ -1416,7 +1409,7 @@
       <c r="C7" s="11" t="n"/>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>Kapı tam açıkken trigger ucunda 12V bulunur ve fotosel 12 beam (geniş algılama alanı) modundadır. MUX B-A (31) full açık sinyali aktif okunur.</t>
+          <t>Kapı tam açıkken röle çeker ve MUX B-A (31) full açık sinyali aktif okunur. Trigger ucunda 12V bulunur ve fotosel 12 beam (geniş algılama alanı) modundadır.</t>
         </is>
       </c>
       <c r="E7" s="11" t="n"/>
@@ -1490,7 +1483,7 @@
       <c r="C10" s="18" t="n"/>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Kapı butonuna basılarak kapı kapatılır; MUX C-C (16) çıkışı, MUX C-A (12) girişi ve kapı hareketi eş zamanlı kaydedilir.</t>
+          <t>Kapı kapatılır; MUX B-A (31) girişi, MUX C-C (16) çıkışı, trigger ucu ve kapı hareketi eş zamanlı kaydedilir.</t>
         </is>
       </c>
       <c r="E10" s="18" t="n"/>
@@ -1516,7 +1509,7 @@
       <c r="C11" s="11" t="n"/>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>Kapı kapanmaya başladığı an 12V kesilir ve fotosel 2 beam (dar algılama alanı) moduna geçer. Kapı kanatları fotoseli tetiklemez; kapı durdurulmadan tam kapalı konuma ulaşır.</t>
+          <t>Kapı tam açık konumdan çıktığı an full açık sinyali düşer, 12V kesilir ve trigger ucu 0V olur; fotosel 2 beam (dar algılama alanı) moduna geçer. Kapı kanatları fotoseli tetiklemez ve kapı durdurulmadan tam kapalı konuma ulaşır.</t>
         </is>
       </c>
       <c r="E11" s="11" t="n"/>

</xml_diff>

<commit_message>
JEST: MUX giris/cikis seviyeleri islendi, KTP detaylandirildi
Seviye tanimlari gereksinimlere ve kabul kriterlerine girdi:
  C MUX A11 analog — 8V ustu = buton basili
  C MUX A12 analog — 8V ustu = engel algilandi
  C MUX B1  dijital — TRUE = TENU C3'e kapi sikisma bilgisi
  C MUX C16 analog/PWM — TRUE = PWM 250 (trigger 12V), FALSE = PWM 0 (0V)
  B MUX A31 analog TERS MANTIK — < 0,5V = kapi full acik

KTP 7 -> 12 madde; her maddenin kabul kriteri olculebilir gerilim degeri
iceriyor ve olculen degerlerin forma kaydedilmesi isteniyor.

Iki yeni acik nokta: PWM frekansinin ve trigger ucundaki ortalama
gerilimin dogrulanmasi, B-A (31) ters mantiginin yazilimda karistirilmamasi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1jP1JN4GEcVEbhfkZatnJ
</commit_message>
<xml_diff>
--- a/JEST_SOFTWARE_KTP_Guncel.xlsx
+++ b/JEST_SOFTWARE_KTP_Guncel.xlsx
@@ -687,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -753,9 +753,9 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>1. MUX C-A (11) ← fotosel ve autoclose ortak butonunun çıkışından muxa giden pin
-2. Bu giriş aktif okunduğunda fotosel fonksiyonu devrededir ve autoclose fonksiyonunun iki koşulundan biri sağlanmış olur.
-3. Giriş pasif okunduğunda MUX engel değerlendirmesi yapmaz ve autoclose aktif olmaz.</t>
+          <t>1. MUX C-A (11) — Analog giriş. 8V üstü okunduğunda fotosel/autoclose butonu BASILI (fonksiyon aktif); 8V altı okunduğunda BIRAKILMIŞ (fonksiyon deaktif).
+2. Giriş 8V üstü okunduğunda fotosel fonksiyonu devrededir ve autoclose fonksiyonunun iki koşulundan biri sağlanmış olur.
+3. Giriş 8V altı okunduğunda MUX engel değerlendirmesi yapmaz ve autoclose aktif olmaz.</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
@@ -782,11 +782,11 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>1. MUX B-A (31) ← kapı full açık sinyali (TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır)
-2. MUX C-C (16) → fotosel trigger ucuna 12V kapı açık sinyali veren çıkış
-3. Kapı full açık → çıkış aktif, trigger ucunda 12V → 12 beam (geniş algılama alanı).
-4. Kapı tam açık konumundan çıktığı an → full açık sinyali düşer, çıkış pasife alınır, trigger ucu 0V → 2 beam (dar algılama alanı).
-5. Kapı kapalı konumdayken ve kapı açılırken çıkış pasif tutulur; kapı tam açık konuma ulaştığında yeniden aktif edilir.
+          <t>1. MUX B-A (31) — Analog giriş, TERS MANTIK. 0,5V (500 mV) ALTI okunduğunda kapı FULL AÇIK; 0,5V ÜSTÜ okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+2. MUX C-C (16) — Analog (PWM) çıkış. TRUE durumunda PWM 250 sürülür ve fotosel trigger ucunda 12V oluşur; FALSE durumunda PWM 0 sürülür ve trigger ucu 0V olur.
+3. MUX B-A (31) &lt; 0,5V (kapı full açık) → MUX C-C (16) TRUE, PWM 250, trigger ucunda 12V → 12 beam (geniş algılama alanı).
+4. MUX B-A (31) &gt; 0,5V (kapı full açık değil) → MUX C-C (16) FALSE, PWM 0, trigger ucu 0V → 2 beam (dar algılama alanı).
+5. Kapı kapalı konumdayken ve kapı açılırken çıkış FALSE tutulur; kapı tam açık konuma ulaştığında yeniden TRUE yapılır.
 6. Röle bobini TENU ön kanat tam açık çıkışına bağlanır; röle kontağının çıkışı MUX B-A (31) girişine verilir.</t>
         </is>
       </c>
@@ -814,9 +814,10 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>1. MUX C-A (12) ← fotoselin engel algılayıp algılamadığının muxa giden pini (Fotosel Output)
-2. Engel algılandığında: MUX C-B (1) → MUX'tan TENU C3'e engel algılanıp algılanmadığı bilgisinin gönderilmesi
-3. Bu bilgi TENU C3 (kapı sıkışma / emniyet fitili) girişine gönderilir; ünite kapıyı durdurur ve geri açar.</t>
+          <t>1. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.
+2. MUX C-A (12) &gt; 8V (engel var) → MUX C-B (1) TRUE yapılır.
+3. MUX C-B (1) — Dijital çıkış. TRUE gönderildiğinde TENU C3'e kapı sıkışma bilgisi iletilir; FALSE'ta hat serbest bırakılır.
+4. Bu bilgi TENU C3 (kapı sıkışma / emniyet fitili) girişine gönderilir; ünite kapıyı durdurur ve geri açar.</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -843,8 +844,8 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>1. MUX C-A (12) ← fotoselin engel algılayıp algılamadığının muxa giden pini (Fotosel Output) pasife döndüğünde MUX C-B (1) çıkışı pasife alınır.
-2. Çıkış pasifken TENU C3 hattı üzerinde herhangi bir yük oluşturmaz; gerçek emniyet fitilinin çalışması etkilenmemelidir.</t>
+          <t>1. MUX C-A (12) &lt; 8V (engel yok) → MUX C-B (1) FALSE yapılır.
+2. Çıkış FALSE iken TENU C3 hattı üzerinde herhangi bir yük oluşturmaz; gerçek emniyet fitilinin çalışması etkilenmemelidir.</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -872,7 +873,7 @@
       <c r="D7" s="5" t="inlineStr">
         <is>
           <t>1. Cluster autoclose seçimi (deaktif dahil) fotosel fonksiyonunu etkilemez.
-2. Koşul yalnızca buton hattının aktif okunmasıdır: MUX C-A (11) ← fotosel ve autoclose ortak butonunun çıkışından muxa giden pin</t>
+2. Koşul yalnızca buton hattının 8V üstü okunmasıdır: MUX C-A (11) — Analog giriş. 8V üstü okunduğunda fotosel/autoclose butonu BASILI (fonksiyon aktif); 8V altı okunduğunda BIRAKILMIŞ (fonksiyon deaktif).</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -900,7 +901,7 @@
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>1. Acil durumda araç yazılımı kapatma komutu vermez.
-2. Acil durum sona erdiğinde engel hâlâ mevcutsa MUX C-B (1) çıkışı yeniden aktif edilir.</t>
+2. Acil durum sona erdiğinde MUX C-A (12) hâlâ 8V üstündeyse MUX C-B (1) çıkışı yeniden TRUE yapılır.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -928,7 +929,7 @@
       <c r="D9" s="5" t="inlineStr">
         <is>
           <t>1. Cluster → araç yazılımına CAN mesajı (seçilen autoclose süresi) — seçilen süre 3 / 10 / 14 olmalıdır (0 = deaktif).
-2. MUX C-A (11) ← fotosel ve autoclose ortak butonunun çıkışından muxa giden pin — aktif okunmalıdır.</t>
+2. MUX C-A (11) — Analog giriş. 8V üstü okunduğunda fotosel/autoclose butonu BASILI (fonksiyon aktif); 8V altı okunduğunda BIRAKILMIŞ (fonksiyon deaktif). — 8V üstü okunmalıdır.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -957,8 +958,10 @@
         <is>
           <t>1. Cluster, araç yazılımına 10 saniye olarak setleme bilgisi gönderir.
 2. Ekranda Telltale 1 aktif edilir.
-3. Sayaç başlangıcı: MUX B-A (31) ← kapı full açık sinyali (TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır)
-4. Sayaç reset: MUX C-A (12) ← fotoselin engel algılayıp algılamadığının muxa giden pini (Fotosel Output) aktif olduğunda.</t>
+3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
+4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
+5. MUX B-A (31) — Analog giriş, TERS MANTIK. 0,5V (500 mV) ALTI okunduğunda kapı FULL AÇIK; 0,5V ÜSTÜ okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+6. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -987,8 +990,10 @@
         <is>
           <t>1. Cluster, araç yazılımına 14 saniye olarak setleme bilgisi gönderir.
 2. Ekranda Telltale 2 aktif edilir.
-3. Sayaç başlangıcı: MUX B-A (31) ← kapı full açık sinyali (TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır)
-4. Sayaç reset: MUX C-A (12) ← fotoselin engel algılayıp algılamadığının muxa giden pini (Fotosel Output) aktif olduğunda.</t>
+3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
+4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
+5. MUX B-A (31) — Analog giriş, TERS MANTIK. 0,5V (500 mV) ALTI okunduğunda kapı FULL AÇIK; 0,5V ÜSTÜ okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+6. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -1017,8 +1022,10 @@
         <is>
           <t>1. Cluster, araç yazılımına 3 saniye olarak setleme bilgisi gönderir.
 2. Ekranda Telltale 3 aktif edilir.
-3. Sayaç başlangıcı: MUX B-A (31) ← kapı full açık sinyali (TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır)
-4. Sayaç reset: MUX C-A (12) ← fotoselin engel algılayıp algılamadığının muxa giden pini (Fotosel Output) aktif olduğunda.</t>
+3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
+4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
+5. MUX B-A (31) — Analog giriş, TERS MANTIK. 0,5V (500 mV) ALTI okunduğunda kapı FULL AÇIK; 0,5V ÜSTÜ okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+6. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1073,7 +1080,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>1. MUX C-A (11) ← fotosel ve autoclose ortak butonunun çıkışından muxa giden pin pasif okunduğunda autoclose fonksiyonu aktif olmaz.
+          <t>1. MUX C-A (11) 8V altı okunduğunda autoclose fonksiyonu aktif olmaz.
 2. Koşullar yeniden sağlandığında fonksiyon normal çalışmasına döner.</t>
         </is>
       </c>
@@ -1203,13 +1210,29 @@
     <row r="23" ht="42" customHeight="1">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>3) Fotosel çıkış seviyesi 12V'tur. MUX C-A (12) girişinin bu seviyeyi dijital giriş olarak doğru okuduğu araç üzerinde doğrulanmalıdır.</t>
+          <t>3) MUX C-C (16) çıkışı PWM ile sürülmektedir (TRUE = PWM 250, FALSE = PWM 0). PWM frekansı ve fotosel trigger girişinde oluşan ortalama gerilim ile dalgalanma araç üzerinde ölçülerek doğrulanmalıdır; trigger girişi seviye bekliyorsa PWM'in sürekli 12V gibi algılandığı teyit edilmelidir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="42" customHeight="1">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>4) MUX B-A (31) girişi TERS MANTIKTA çalışır: düşük gerilim (&lt; 0,5V) kapı full açık, yüksek gerilim kapı full açık değil demektir. Yazılımda bu yön karıştırılmamalıdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>5) Fotosel çıkış seviyesi 12V'tur. MUX C-A (12) girişinin bu seviyeyi dijital giriş olarak doğru okuduğu araç üzerinde doğrulanmalıdır.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A25:E25"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A22:E22"/>
@@ -1226,7 +1249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1283,7 +1306,7 @@
       <c r="C2" s="18" t="n"/>
       <c r="D2" s="19" t="inlineStr">
         <is>
-          <t>Buton aktif konuma getirilir; MUX C-A (11) girişi ve fotosel besleme hattı ölçülür. Ardından buton bırakılır.</t>
+          <t>Fotosel/autoclose butonu basılı konuma getirilir ve MUX C-A (11) analog girişi ölçülür. Ardından buton bırakılır ve ölçüm tekrarlanır. Her iki konumda fotoselin besleme hattı da kontrol edilir.</t>
         </is>
       </c>
       <c r="E2" s="18" t="n"/>
@@ -1309,7 +1332,7 @@
       <c r="C3" s="11" t="n"/>
       <c r="D3" s="23" t="inlineStr">
         <is>
-          <t>Buton aktifken MUX C-A (11) girişi aktif okunur ve fotosel beslemededir. Buton bırakıldığında giriş pasif okunur, fotosel beslemesiz kalır ve kapı normal çalışır.</t>
+          <t>Buton basılıyken MUX C-A (11) girişinde 8V ÜSTÜ değer okunmalı ve fotosel beslemede olmalıdır. Buton bırakıldığında 8V ALTI değer okunmalı ve fotosel beslemesiz kalmalıdır. Okunan gerilim değerleri bu forma kaydedilmelidir.</t>
         </is>
       </c>
       <c r="E3" s="11" t="n"/>
@@ -1383,7 +1406,7 @@
       <c r="C6" s="18" t="n"/>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Kapı tam açık konuma getirilir; TENU ön kanat tam açık çıkışı, röle kontağı, MUX B-A (31) girişi, MUX C-C (16) çıkışı ve fotosel trigger ucu birlikte ölçülür.</t>
+          <t>Buton basılı konumdayken fotosel enerjilendirilir; gösterge LED'leri ve ilk enerjilenme davranışı gözlenir. Fotosel önüne engel konulup kaldırılarak MUX C-A (12) analog girişi izlenir.</t>
         </is>
       </c>
       <c r="E6" s="18" t="n"/>
@@ -1409,7 +1432,7 @@
       <c r="C7" s="11" t="n"/>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>Kapı tam açıkken röle çeker ve MUX B-A (31) full açık sinyali aktif okunur. Trigger ucunda 12V bulunur ve fotosel 12 beam (geniş algılama alanı) modundadır.</t>
+          <t>Engel konulduğunda MUX C-A (12) girişinde 8V ÜSTÜ değer okunmalı, engel kaldırıldığında 8V ALTI değere dönmelidir. Okunan gerilim değerleri bu forma kaydedilmelidir.</t>
         </is>
       </c>
       <c r="E7" s="11" t="n"/>
@@ -1483,7 +1506,7 @@
       <c r="C10" s="18" t="n"/>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Kapı kapatılır; MUX B-A (31) girişi, MUX C-C (16) çıkışı, trigger ucu ve kapı hareketi eş zamanlı kaydedilir.</t>
+          <t>Kapı tam açık konuma getirilir. TENU ön kanat tam açık çıkışı, röle kontağı, MUX B-A (31) analog girişi, MUX C-C (16) çıkışı ve fotosel trigger ucu birlikte ölçülür.</t>
         </is>
       </c>
       <c r="E10" s="18" t="n"/>
@@ -1509,7 +1532,7 @@
       <c r="C11" s="11" t="n"/>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>Kapı tam açık konumdan çıktığı an full açık sinyali düşer, 12V kesilir ve trigger ucu 0V olur; fotosel 2 beam (dar algılama alanı) moduna geçer. Kapı kanatları fotoseli tetiklemez ve kapı durdurulmadan tam kapalı konuma ulaşır.</t>
+          <t>Kapı tam açıkken röle çekmeli ve MUX B-A (31) girişinde 0,5V ALTI (&lt; 500 mV) değer okunmalıdır. Araç yazılımı MUX C-C (16) çıkışını TRUE yaparak PWM 250 sürmeli, fotosel trigger ucunda 12V ölçülmelidir. Fotosel 12 beam (geniş algılama alanı) modunda olmalıdır. Ölçülen değerler bu forma kaydedilmelidir.</t>
         </is>
       </c>
       <c r="E11" s="11" t="n"/>
@@ -1583,7 +1606,7 @@
       <c r="C14" s="18" t="n"/>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Kapı açıkken fotosel önüne engel konur ve kapatma isteği gönderilir. Ardından engel kaldırılır.</t>
+          <t>Kapı tam açık konumdan çıkarılır (kapanmaya başlatılır). MUX B-A (31) girişi, MUX C-C (16) çıkışı ve fotosel trigger ucu eş zamanlı kaydedilir.</t>
         </is>
       </c>
       <c r="E14" s="18" t="n"/>
@@ -1609,7 +1632,7 @@
       <c r="C15" s="11" t="n"/>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>MUX C-A (12) aktif okunur ve MUX C-B (1) çıkışı sürülür; TENU C3 üzerinden kapı kapatılmaz, kapanmakta ise durdurulup geri açılır. Engel kaldırıldığında çıkış pasife alınır ve kapatma isteği tekrar kabul edilir.</t>
+          <t>Kapı tam açık konumdan çıktığı anda MUX B-A (31) girişinde 0,5V ÜSTÜ değer okunmalı, MUX C-C (16) çıkışı FALSE olmalı (PWM 0) ve trigger ucu 0V'a düşmelidir. Fotosel 2 beam (dar algılama alanı) moduna geçmelidir. Geçiş, kanatların ışın alanına girmesinden ÖNCE tamamlanmalıdır.</t>
         </is>
       </c>
       <c r="E15" s="11" t="n"/>
@@ -1683,7 +1706,7 @@
       <c r="C18" s="18" t="n"/>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Cluster üzerinden sırasıyla 10 sn, 14 sn, 3 sn ve deaktif seçilir; her seçimde buton aktif, kapı tam açık konuma getirilerek engelsiz beklenir.</t>
+          <t>Fotosel önünde engel bulunmadan kapı tam açıktan tam kapalıya kadar kapatılır. MUX C-A (12) girişi kapanma boyunca kaydedilir.</t>
         </is>
       </c>
       <c r="E18" s="18" t="n"/>
@@ -1709,7 +1732,7 @@
       <c r="C19" s="11" t="n"/>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t>Her seçimde ilgili telltale görüntülenir ve kapı seçili süre sonunda kapanır. Deaktif seçiliyken telltale görüntülenmez ve kapı kendiliğinden kapanmaz.</t>
+          <t>Kapanma boyunca MUX C-A (12) girişi 8V ALTINDA kalmalı; kapı kanatları fotoseli tetiklememelidir. Kapı durdurulmadan, kesintisiz olarak tam kapalı konuma ulaşmalıdır.</t>
         </is>
       </c>
       <c r="E19" s="11" t="n"/>
@@ -1783,7 +1806,7 @@
       <c r="C22" s="18" t="n"/>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Auto Close 10 sn seçiliyken sayaç çalışırken fotosele engel verilir, ardından engel kaldırılır.</t>
+          <t>Kapı açıkken fotosel önüne engel konur ve kapatma isteği gönderilir. MUX C-A (12) girişi, MUX C-B (1) çıkışı, TENU C3 hattı ve kapı hareketi izlenir.</t>
         </is>
       </c>
       <c r="E22" s="18" t="n"/>
@@ -1809,7 +1832,7 @@
       <c r="C23" s="11" t="n"/>
       <c r="D23" s="23" t="inlineStr">
         <is>
-          <t>Sayaç sıfırlanır. Kapı ancak engel kalktıktan sonra kesintisiz 10 saniye geçince kapanır.</t>
+          <t>MUX C-A (12) girişinde 8V ÜSTÜ değer okunmalı, MUX C-B (1) çıkışı TRUE olmalı ve TENU C3 hattına kapı sıkışma bilgisi iletilmelidir. Kapı kapanmamalı; kapanmakta ise durdurulup geri açılmalıdır. Komut şoför butonundan, dış butondan veya uzaktan kumandadan gelse dahi kapı kapanmamalıdır.</t>
         </is>
       </c>
       <c r="E23" s="11" t="n"/>
@@ -1883,7 +1906,7 @@
       <c r="C26" s="18" t="n"/>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>Sayaç çalışırken sırasıyla acil durum, yangın algılama (MUX E (A) 18 / E (A) 17) ve blokaj butonu (MUX C (A) 16 / C (A) 23) aktif edilir; her biri ayrı ayrı denenip kaldırılır.</t>
+          <t>Engel kaldırılır. MUX C-A (12) girişi, MUX C-B (1) çıkışı ve TENU C3 hattı izlenir. Ardından gerçek emniyet fitiline elle basılarak kapı kontrol ünitesinin tepkisi kontrol edilir.</t>
         </is>
       </c>
       <c r="E26" s="18" t="n"/>
@@ -1909,7 +1932,7 @@
       <c r="C27" s="11" t="n"/>
       <c r="D27" s="23" t="inlineStr">
         <is>
-          <t>Her üç durumda da sayaç durur ve kapı kapatma komutu verilmez. Durum kalktığında sayaç yeniden başlar ve kapı seçili süre sonunda kapanır.</t>
+          <t>Engel kalktığında MUX C-A (12) 8V ALTINA inmeli, MUX C-B (1) çıkışı FALSE olmalı ve TENU C3 hattı serbest bırakılmalıdır; kapatma isteği tekrar kabul edilmelidir. Çıkış FALSE iken hat üzerinde yük oluşturmamalı, gerçek emniyet fitilinin çalışması etkilenmemelidir.</t>
         </is>
       </c>
       <c r="E27" s="11" t="n"/>
@@ -1969,72 +1992,617 @@
       <c r="O29" s="27" t="n"/>
       <c r="P29" s="29" t="n"/>
     </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>MADDE 8 :</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>PROSEDÜR</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Cluster üzerinden sırasıyla 10 sn, 14 sn ve 3 sn seçilir. Her seçimde buton basılı, kapı tam açık konuma getirilerek engelsiz beklenir ve kapanma süresi kronometre ile ölçülür.</t>
+        </is>
+      </c>
+      <c r="E30" s="18" t="n"/>
+      <c r="F30" s="18" t="n"/>
+      <c r="G30" s="18" t="n"/>
+      <c r="H30" s="18" t="n"/>
+      <c r="I30" s="18" t="n"/>
+      <c r="J30" s="18" t="n"/>
+      <c r="K30" s="18" t="n"/>
+      <c r="L30" s="18" t="n"/>
+      <c r="M30" s="18" t="n"/>
+      <c r="N30" s="18" t="n"/>
+      <c r="O30" s="18" t="n"/>
+      <c r="P30" s="20" t="n"/>
+    </row>
+    <row r="31" ht="36" customHeight="1">
+      <c r="A31" s="21" t="n"/>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>KABUL KRİTERİ</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="23" t="inlineStr">
+        <is>
+          <t>Her seçimde ekranda ilgili telltale görüntülenmelidir (10 sn → Telltale 1, 14 sn → Telltale 2, 3 sn → Telltale 3). Geri sayım, MUX B-A (31) girişi 0,5V altına indiği anda başlamalı ve kapı seçili süre sonunda kapanmalıdır. Ölçülen süreler bu forma kaydedilmelidir.</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="11" t="n"/>
+      <c r="I31" s="11" t="n"/>
+      <c r="J31" s="11" t="n"/>
+      <c r="K31" s="11" t="n"/>
+      <c r="L31" s="11" t="n"/>
+      <c r="M31" s="11" t="n"/>
+      <c r="N31" s="11" t="n"/>
+      <c r="O31" s="11" t="n"/>
+      <c r="P31" s="24" t="n"/>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="21" t="n"/>
+      <c r="B32" s="22" t="inlineStr">
+        <is>
+          <t>SONUÇ</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="n"/>
+      <c r="D32" s="23" t="inlineStr"/>
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="11" t="n"/>
+      <c r="G32" s="11" t="n"/>
+      <c r="H32" s="11" t="n"/>
+      <c r="I32" s="11" t="n"/>
+      <c r="J32" s="11" t="n"/>
+      <c r="K32" s="11" t="n"/>
+      <c r="L32" s="11" t="n"/>
+      <c r="M32" s="11" t="n"/>
+      <c r="N32" s="11" t="n"/>
+      <c r="O32" s="11" t="n"/>
+      <c r="P32" s="24" t="n"/>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="25" t="n"/>
+      <c r="B33" s="26" t="inlineStr">
+        <is>
+          <t>OK / NOK</t>
+        </is>
+      </c>
+      <c r="C33" s="27" t="n"/>
+      <c r="D33" s="28" t="inlineStr"/>
+      <c r="E33" s="27" t="n"/>
+      <c r="F33" s="27" t="n"/>
+      <c r="G33" s="27" t="n"/>
+      <c r="H33" s="27" t="n"/>
+      <c r="I33" s="27" t="n"/>
+      <c r="J33" s="27" t="n"/>
+      <c r="K33" s="27" t="n"/>
+      <c r="L33" s="27" t="n"/>
+      <c r="M33" s="27" t="n"/>
+      <c r="N33" s="27" t="n"/>
+      <c r="O33" s="27" t="n"/>
+      <c r="P33" s="29" t="n"/>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>MADDE 9 :</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>PROSEDÜR</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="n"/>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>Auto Close 10 sn seçiliyken sayaç çalışırken fotosel önüne engel konur, bir süre bekletilip kaldırılır.</t>
+        </is>
+      </c>
+      <c r="E34" s="18" t="n"/>
+      <c r="F34" s="18" t="n"/>
+      <c r="G34" s="18" t="n"/>
+      <c r="H34" s="18" t="n"/>
+      <c r="I34" s="18" t="n"/>
+      <c r="J34" s="18" t="n"/>
+      <c r="K34" s="18" t="n"/>
+      <c r="L34" s="18" t="n"/>
+      <c r="M34" s="18" t="n"/>
+      <c r="N34" s="18" t="n"/>
+      <c r="O34" s="18" t="n"/>
+      <c r="P34" s="20" t="n"/>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="21" t="n"/>
+      <c r="B35" s="22" t="inlineStr">
+        <is>
+          <t>KABUL KRİTERİ</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="n"/>
+      <c r="D35" s="23" t="inlineStr">
+        <is>
+          <t>MUX C-A (12) 8V üstüne çıktığında sayaç sıfırlanmalıdır. Kapı ancak engel kalktıktan sonra kesintisiz 10 saniye geçince kapanmalıdır.</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="n"/>
+      <c r="F35" s="11" t="n"/>
+      <c r="G35" s="11" t="n"/>
+      <c r="H35" s="11" t="n"/>
+      <c r="I35" s="11" t="n"/>
+      <c r="J35" s="11" t="n"/>
+      <c r="K35" s="11" t="n"/>
+      <c r="L35" s="11" t="n"/>
+      <c r="M35" s="11" t="n"/>
+      <c r="N35" s="11" t="n"/>
+      <c r="O35" s="11" t="n"/>
+      <c r="P35" s="24" t="n"/>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="21" t="n"/>
+      <c r="B36" s="22" t="inlineStr">
+        <is>
+          <t>SONUÇ</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="n"/>
+      <c r="D36" s="23" t="inlineStr"/>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="11" t="n"/>
+      <c r="G36" s="11" t="n"/>
+      <c r="H36" s="11" t="n"/>
+      <c r="I36" s="11" t="n"/>
+      <c r="J36" s="11" t="n"/>
+      <c r="K36" s="11" t="n"/>
+      <c r="L36" s="11" t="n"/>
+      <c r="M36" s="11" t="n"/>
+      <c r="N36" s="11" t="n"/>
+      <c r="O36" s="11" t="n"/>
+      <c r="P36" s="24" t="n"/>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="25" t="n"/>
+      <c r="B37" s="26" t="inlineStr">
+        <is>
+          <t>OK / NOK</t>
+        </is>
+      </c>
+      <c r="C37" s="27" t="n"/>
+      <c r="D37" s="28" t="inlineStr"/>
+      <c r="E37" s="27" t="n"/>
+      <c r="F37" s="27" t="n"/>
+      <c r="G37" s="27" t="n"/>
+      <c r="H37" s="27" t="n"/>
+      <c r="I37" s="27" t="n"/>
+      <c r="J37" s="27" t="n"/>
+      <c r="K37" s="27" t="n"/>
+      <c r="L37" s="27" t="n"/>
+      <c r="M37" s="27" t="n"/>
+      <c r="N37" s="27" t="n"/>
+      <c r="O37" s="27" t="n"/>
+      <c r="P37" s="29" t="n"/>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>MADDE 10 :</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>PROSEDÜR</t>
+        </is>
+      </c>
+      <c r="C38" s="18" t="n"/>
+      <c r="D38" s="19" t="inlineStr">
+        <is>
+          <t>Cluster üzerinden autoclose deaktif seçilir; kapı tam açık konuma getirilip 20 saniyeden uzun süre beklenir. Ardından buton bırakılmış durumda 10 sn seçilerek aynı bekleme tekrarlanır.</t>
+        </is>
+      </c>
+      <c r="E38" s="18" t="n"/>
+      <c r="F38" s="18" t="n"/>
+      <c r="G38" s="18" t="n"/>
+      <c r="H38" s="18" t="n"/>
+      <c r="I38" s="18" t="n"/>
+      <c r="J38" s="18" t="n"/>
+      <c r="K38" s="18" t="n"/>
+      <c r="L38" s="18" t="n"/>
+      <c r="M38" s="18" t="n"/>
+      <c r="N38" s="18" t="n"/>
+      <c r="O38" s="18" t="n"/>
+      <c r="P38" s="20" t="n"/>
+    </row>
+    <row r="39" ht="36" customHeight="1">
+      <c r="A39" s="21" t="n"/>
+      <c r="B39" s="22" t="inlineStr">
+        <is>
+          <t>KABUL KRİTERİ</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="23" t="inlineStr">
+        <is>
+          <t>Her iki durumda da ekranda autoclose telltale'i görüntülenmemeli ve kapı kendiliğinden kapanmamalıdır. Fotosel fonksiyonu (engel algılandığında kapının kapanmaması) çalışmaya devam etmelidir.</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="11" t="n"/>
+      <c r="G39" s="11" t="n"/>
+      <c r="H39" s="11" t="n"/>
+      <c r="I39" s="11" t="n"/>
+      <c r="J39" s="11" t="n"/>
+      <c r="K39" s="11" t="n"/>
+      <c r="L39" s="11" t="n"/>
+      <c r="M39" s="11" t="n"/>
+      <c r="N39" s="11" t="n"/>
+      <c r="O39" s="11" t="n"/>
+      <c r="P39" s="24" t="n"/>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="21" t="n"/>
+      <c r="B40" s="22" t="inlineStr">
+        <is>
+          <t>SONUÇ</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="n"/>
+      <c r="D40" s="23" t="inlineStr"/>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="11" t="n"/>
+      <c r="G40" s="11" t="n"/>
+      <c r="H40" s="11" t="n"/>
+      <c r="I40" s="11" t="n"/>
+      <c r="J40" s="11" t="n"/>
+      <c r="K40" s="11" t="n"/>
+      <c r="L40" s="11" t="n"/>
+      <c r="M40" s="11" t="n"/>
+      <c r="N40" s="11" t="n"/>
+      <c r="O40" s="11" t="n"/>
+      <c r="P40" s="24" t="n"/>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="25" t="n"/>
+      <c r="B41" s="26" t="inlineStr">
+        <is>
+          <t>OK / NOK</t>
+        </is>
+      </c>
+      <c r="C41" s="27" t="n"/>
+      <c r="D41" s="28" t="inlineStr"/>
+      <c r="E41" s="27" t="n"/>
+      <c r="F41" s="27" t="n"/>
+      <c r="G41" s="27" t="n"/>
+      <c r="H41" s="27" t="n"/>
+      <c r="I41" s="27" t="n"/>
+      <c r="J41" s="27" t="n"/>
+      <c r="K41" s="27" t="n"/>
+      <c r="L41" s="27" t="n"/>
+      <c r="M41" s="27" t="n"/>
+      <c r="N41" s="27" t="n"/>
+      <c r="O41" s="27" t="n"/>
+      <c r="P41" s="29" t="n"/>
+    </row>
+    <row r="42" ht="32" customHeight="1">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>MADDE 11 :</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="inlineStr">
+        <is>
+          <t>PROSEDÜR</t>
+        </is>
+      </c>
+      <c r="C42" s="18" t="n"/>
+      <c r="D42" s="19" t="inlineStr">
+        <is>
+          <t>Sayaç çalışırken sırasıyla acil durum, yangın algılama (MUX E (A) 18 GND / MUX E (A) 17 12V) ve blokaj butonu (MUX C (A) 16 / MUX C (A) 23) aktif edilir; her biri ayrı ayrı denenip kaldırılır.</t>
+        </is>
+      </c>
+      <c r="E42" s="18" t="n"/>
+      <c r="F42" s="18" t="n"/>
+      <c r="G42" s="18" t="n"/>
+      <c r="H42" s="18" t="n"/>
+      <c r="I42" s="18" t="n"/>
+      <c r="J42" s="18" t="n"/>
+      <c r="K42" s="18" t="n"/>
+      <c r="L42" s="18" t="n"/>
+      <c r="M42" s="18" t="n"/>
+      <c r="N42" s="18" t="n"/>
+      <c r="O42" s="18" t="n"/>
+      <c r="P42" s="20" t="n"/>
+    </row>
+    <row r="43" ht="36" customHeight="1">
+      <c r="A43" s="21" t="n"/>
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>KABUL KRİTERİ</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="n"/>
+      <c r="D43" s="23" t="inlineStr">
+        <is>
+          <t>Her üç durumda da sayaç durmalı ve kapı kapatma komutu verilmemelidir. Durum kalktığında sayaç yeniden başlamalı ve kapı seçili süre sonunda kapanmalıdır.</t>
+        </is>
+      </c>
+      <c r="E43" s="11" t="n"/>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="11" t="n"/>
+      <c r="H43" s="11" t="n"/>
+      <c r="I43" s="11" t="n"/>
+      <c r="J43" s="11" t="n"/>
+      <c r="K43" s="11" t="n"/>
+      <c r="L43" s="11" t="n"/>
+      <c r="M43" s="11" t="n"/>
+      <c r="N43" s="11" t="n"/>
+      <c r="O43" s="11" t="n"/>
+      <c r="P43" s="24" t="n"/>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="21" t="n"/>
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>SONUÇ</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="n"/>
+      <c r="D44" s="23" t="inlineStr"/>
+      <c r="E44" s="11" t="n"/>
+      <c r="F44" s="11" t="n"/>
+      <c r="G44" s="11" t="n"/>
+      <c r="H44" s="11" t="n"/>
+      <c r="I44" s="11" t="n"/>
+      <c r="J44" s="11" t="n"/>
+      <c r="K44" s="11" t="n"/>
+      <c r="L44" s="11" t="n"/>
+      <c r="M44" s="11" t="n"/>
+      <c r="N44" s="11" t="n"/>
+      <c r="O44" s="11" t="n"/>
+      <c r="P44" s="24" t="n"/>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="25" t="n"/>
+      <c r="B45" s="26" t="inlineStr">
+        <is>
+          <t>OK / NOK</t>
+        </is>
+      </c>
+      <c r="C45" s="27" t="n"/>
+      <c r="D45" s="28" t="inlineStr"/>
+      <c r="E45" s="27" t="n"/>
+      <c r="F45" s="27" t="n"/>
+      <c r="G45" s="27" t="n"/>
+      <c r="H45" s="27" t="n"/>
+      <c r="I45" s="27" t="n"/>
+      <c r="J45" s="27" t="n"/>
+      <c r="K45" s="27" t="n"/>
+      <c r="L45" s="27" t="n"/>
+      <c r="M45" s="27" t="n"/>
+      <c r="N45" s="27" t="n"/>
+      <c r="O45" s="27" t="n"/>
+      <c r="P45" s="29" t="n"/>
+    </row>
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>MADDE 12 :</t>
+        </is>
+      </c>
+      <c r="B46" s="17" t="inlineStr">
+        <is>
+          <t>PROSEDÜR</t>
+        </is>
+      </c>
+      <c r="C46" s="18" t="n"/>
+      <c r="D46" s="19" t="inlineStr">
+        <is>
+          <t>Fotosel sinyal hattı (MUX C-A 12) sökülerek geçersiz duruma getirilir, ardından geri bağlanır. Aynı işlem MUX B-A (31) full açık sinyal hattı için tekrarlanır.</t>
+        </is>
+      </c>
+      <c r="E46" s="18" t="n"/>
+      <c r="F46" s="18" t="n"/>
+      <c r="G46" s="18" t="n"/>
+      <c r="H46" s="18" t="n"/>
+      <c r="I46" s="18" t="n"/>
+      <c r="J46" s="18" t="n"/>
+      <c r="K46" s="18" t="n"/>
+      <c r="L46" s="18" t="n"/>
+      <c r="M46" s="18" t="n"/>
+      <c r="N46" s="18" t="n"/>
+      <c r="O46" s="18" t="n"/>
+      <c r="P46" s="20" t="n"/>
+    </row>
+    <row r="47" ht="36" customHeight="1">
+      <c r="A47" s="21" t="n"/>
+      <c r="B47" s="22" t="inlineStr">
+        <is>
+          <t>KABUL KRİTERİ</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="n"/>
+      <c r="D47" s="23" t="inlineStr">
+        <is>
+          <t>Araç yazılımı geçersiz seviyeyi tespit etmeli ve kapı kapatma komutu vermemelidir. Hatlar geri bağlandığında fonksiyon normal çalışmasına dönmelidir.</t>
+        </is>
+      </c>
+      <c r="E47" s="11" t="n"/>
+      <c r="F47" s="11" t="n"/>
+      <c r="G47" s="11" t="n"/>
+      <c r="H47" s="11" t="n"/>
+      <c r="I47" s="11" t="n"/>
+      <c r="J47" s="11" t="n"/>
+      <c r="K47" s="11" t="n"/>
+      <c r="L47" s="11" t="n"/>
+      <c r="M47" s="11" t="n"/>
+      <c r="N47" s="11" t="n"/>
+      <c r="O47" s="11" t="n"/>
+      <c r="P47" s="24" t="n"/>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="A48" s="21" t="n"/>
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>SONUÇ</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="n"/>
+      <c r="D48" s="23" t="inlineStr"/>
+      <c r="E48" s="11" t="n"/>
+      <c r="F48" s="11" t="n"/>
+      <c r="G48" s="11" t="n"/>
+      <c r="H48" s="11" t="n"/>
+      <c r="I48" s="11" t="n"/>
+      <c r="J48" s="11" t="n"/>
+      <c r="K48" s="11" t="n"/>
+      <c r="L48" s="11" t="n"/>
+      <c r="M48" s="11" t="n"/>
+      <c r="N48" s="11" t="n"/>
+      <c r="O48" s="11" t="n"/>
+      <c r="P48" s="24" t="n"/>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="25" t="n"/>
+      <c r="B49" s="26" t="inlineStr">
+        <is>
+          <t>OK / NOK</t>
+        </is>
+      </c>
+      <c r="C49" s="27" t="n"/>
+      <c r="D49" s="28" t="inlineStr"/>
+      <c r="E49" s="27" t="n"/>
+      <c r="F49" s="27" t="n"/>
+      <c r="G49" s="27" t="n"/>
+      <c r="H49" s="27" t="n"/>
+      <c r="I49" s="27" t="n"/>
+      <c r="J49" s="27" t="n"/>
+      <c r="K49" s="27" t="n"/>
+      <c r="L49" s="27" t="n"/>
+      <c r="M49" s="27" t="n"/>
+      <c r="N49" s="27" t="n"/>
+      <c r="O49" s="27" t="n"/>
+      <c r="P49" s="29" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="64">
-    <mergeCell ref="D28:P28"/>
+  <mergeCells count="109">
+    <mergeCell ref="D18:P18"/>
+    <mergeCell ref="D3:P3"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="D25:P25"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D5:P5"/>
+    <mergeCell ref="D20:P20"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="D22:P22"/>
+    <mergeCell ref="D31:P31"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="D45:P45"/>
+    <mergeCell ref="D6:P6"/>
+    <mergeCell ref="D21:P21"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D7:P7"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="D16:P16"/>
+    <mergeCell ref="B35:C35"/>
     <mergeCell ref="D4:P4"/>
     <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D18:P18"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D9:P9"/>
-    <mergeCell ref="D12:P12"/>
-    <mergeCell ref="D3:P3"/>
-    <mergeCell ref="B22:C22"/>
     <mergeCell ref="D8:P8"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D15:P15"/>
-    <mergeCell ref="D25:P25"/>
     <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D24:P24"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D14:P14"/>
-    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D33:P33"/>
+    <mergeCell ref="D42:P42"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D5:P5"/>
-    <mergeCell ref="D23:P23"/>
-    <mergeCell ref="D29:P29"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D20:P20"/>
-    <mergeCell ref="D26:P26"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D35:P35"/>
+    <mergeCell ref="D44:P44"/>
     <mergeCell ref="D19:P19"/>
-    <mergeCell ref="D10:P10"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="D22:P22"/>
+    <mergeCell ref="D34:P34"/>
     <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A46:A49"/>
     <mergeCell ref="A1:P1"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D6:P6"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="D21:P21"/>
-    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="D36:P36"/>
     <mergeCell ref="D11:P11"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="D2:P2"/>
-    <mergeCell ref="A22:A25"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="D13:P13"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="D27:P27"/>
     <mergeCell ref="B15:C15"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="D48:P48"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D9:P9"/>
+    <mergeCell ref="D15:P15"/>
+    <mergeCell ref="D24:P24"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="D38:P38"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="D26:P26"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D10:P10"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D49:P49"/>
+    <mergeCell ref="D2:P2"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="D47:P47"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D28:P28"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="D37:P37"/>
+    <mergeCell ref="D12:P12"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="D30:P30"/>
+    <mergeCell ref="D39:P39"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="D14:P14"/>
+    <mergeCell ref="D29:P29"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="D23:P23"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D46:P46"/>
+    <mergeCell ref="D40:P40"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D32:P32"/>
+    <mergeCell ref="D27:P27"/>
+    <mergeCell ref="D41:P41"/>
     <mergeCell ref="D17:P17"/>
-    <mergeCell ref="D7:P7"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="D16:P16"/>
-    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="D43:P43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
JEST: B-A (31) icin 'ters mantik' vurgusu kaldirildi
Esik degerleri oldugu gibi birakildi; ayrica eklenen ters mantik uyarisi
ve ilgili acik nokta notu cikarildi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1jP1JN4GEcVEbhfkZatnJ
</commit_message>
<xml_diff>
--- a/JEST_SOFTWARE_KTP_Guncel.xlsx
+++ b/JEST_SOFTWARE_KTP_Guncel.xlsx
@@ -687,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -782,7 +782,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>1. MUX B-A (31) — Analog giriş, TERS MANTIK. 0,5V (500 mV) ALTI okunduğunda kapı FULL AÇIK; 0,5V ÜSTÜ okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+          <t>1. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
 2. MUX C-C (16) — Analog (PWM) çıkış. TRUE durumunda PWM 250 sürülür ve fotosel trigger ucunda 12V oluşur; FALSE durumunda PWM 0 sürülür ve trigger ucu 0V olur.
 3. MUX B-A (31) &lt; 0,5V (kapı full açık) → MUX C-C (16) TRUE, PWM 250, trigger ucunda 12V → 12 beam (geniş algılama alanı).
 4. MUX B-A (31) &gt; 0,5V (kapı full açık değil) → MUX C-C (16) FALSE, PWM 0, trigger ucu 0V → 2 beam (dar algılama alanı).
@@ -960,7 +960,7 @@
 2. Ekranda Telltale 1 aktif edilir.
 3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
 4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
-5. MUX B-A (31) — Analog giriş, TERS MANTIK. 0,5V (500 mV) ALTI okunduğunda kapı FULL AÇIK; 0,5V ÜSTÜ okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+5. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
 6. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
         </is>
       </c>
@@ -992,7 +992,7 @@
 2. Ekranda Telltale 2 aktif edilir.
 3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
 4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
-5. MUX B-A (31) — Analog giriş, TERS MANTIK. 0,5V (500 mV) ALTI okunduğunda kapı FULL AÇIK; 0,5V ÜSTÜ okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+5. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
 6. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
         </is>
       </c>
@@ -1024,7 +1024,7 @@
 2. Ekranda Telltale 3 aktif edilir.
 3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
 4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
-5. MUX B-A (31) — Analog giriş, TERS MANTIK. 0,5V (500 mV) ALTI okunduğunda kapı FULL AÇIK; 0,5V ÜSTÜ okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+5. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
 6. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
         </is>
       </c>
@@ -1217,22 +1217,14 @@
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>4) MUX B-A (31) girişi TERS MANTIKTA çalışır: düşük gerilim (&lt; 0,5V) kapı full açık, yüksek gerilim kapı full açık değil demektir. Yazılımda bu yön karıştırılmamalıdır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="42" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>5) Fotosel çıkış seviyesi 12V'tur. MUX C-A (12) girişinin bu seviyeyi dijital giriş olarak doğru okuduğu araç üzerinde doğrulanmalıdır.</t>
+          <t>4) Fotosel çıkış seviyesi 12V'tur. MUX C-A (12) girişinin bu seviyeyi dijital giriş olarak doğru okuduğu araç üzerinde doğrulanmalıdır.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="6">
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A25:E25"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A22:E22"/>

</xml_diff>

<commit_message>
JEST: emniyet fitili acik nokta olmaktan cikarildi
Emniyet fitili kapi kontrol unitesinin kendi fonksiyonudur; arac yazilimi
TENU C3 pinine yalnizca giris yapar, hatti okumaz. Sayacin emniyet fitili
ile sifirlanmasini acik nokta olarak yazan not kaldirildi ve kapsam
1.c'de acikca ifade edildi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1jP1JN4GEcVEbhfkZatnJ
</commit_message>
<xml_diff>
--- a/JEST_SOFTWARE_KTP_Guncel.xlsx
+++ b/JEST_SOFTWARE_KTP_Guncel.xlsx
@@ -687,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -845,7 +845,8 @@
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>1. MUX C-A (12) &lt; 8V (engel yok) → MUX C-B (1) FALSE yapılır.
-2. Çıkış FALSE iken TENU C3 hattı üzerinde herhangi bir yük oluşturmaz; gerçek emniyet fitilinin çalışması etkilenmemelidir.</t>
+2. Emniyet fitili kapı kontrol ünitesinin kendi fonksiyonudur; araç yazılımı bu hattı yalnızca sürer, okumaz ve fitilin kendi çalışmasına müdahale etmez.
+3. Çıkış FALSE iken TENU C3 hattı üzerinde herhangi bir yük oluşturmaz; gerçek emniyet fitilinin çalışması etkilenmemelidir.</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1196,35 +1197,27 @@
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>1) Kapı sıkışma (emniyet fitili) bilgisi artık MUX'a giriş olarak gelmemektedir; MUX C-B (1) yalnızca TENU C3'e bilgi gönderen bir çıkıştır. Bu nedenle 2.a / 2.b / 2.c maddelerinde sayaç yalnızca fotosel engel bilgisi ile sıfırlanmaktadır. Sayacın emniyet fitiline basıldığında da sıfırlanması isteniyorsa MUX'a ayrı bir giriş tahsis edilmelidir.</t>
+          <t>1) I/O listesinde kapı kapatma komutuna ait bir çıkış bulunmamaktadır. Autoclose süresi dolduğunda kapının hangi çıkış üzerinden kapatılacağı (TENU B4 kapı butonu hattı veya başka bir yol) netleştirilerek bu tabloya işlenmelidir.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>2) I/O listesinde kapı kapatma komutuna ait bir çıkış bulunmamaktadır. Autoclose süresi dolduğunda kapının hangi çıkış üzerinden kapatılacağı (TENU B4 kapı butonu hattı veya başka bir yol) netleştirilerek bu tabloya işlenmelidir.</t>
+          <t>2) MUX C-C (16) çıkışı PWM ile sürülmektedir (TRUE = PWM 250, FALSE = PWM 0). PWM frekansı ve fotosel trigger girişinde oluşan ortalama gerilim ile dalgalanma araç üzerinde ölçülerek doğrulanmalıdır; trigger girişi seviye bekliyorsa PWM'in sürekli 12V gibi algılandığı teyit edilmelidir.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>3) MUX C-C (16) çıkışı PWM ile sürülmektedir (TRUE = PWM 250, FALSE = PWM 0). PWM frekansı ve fotosel trigger girişinde oluşan ortalama gerilim ile dalgalanma araç üzerinde ölçülerek doğrulanmalıdır; trigger girişi seviye bekliyorsa PWM'in sürekli 12V gibi algılandığı teyit edilmelidir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="42" customHeight="1">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t>4) Fotosel çıkış seviyesi 12V'tur. MUX C-A (12) girişinin bu seviyeyi dijital giriş olarak doğru okuduğu araç üzerinde doğrulanmalıdır.</t>
+          <t>3) Fotosel çıkış seviyesi 12V'tur. MUX C-A (12) girişinin bu seviyeyi dijital giriş olarak doğru okuduğu araç üzerinde doğrulanmalıdır.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A24:E24"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A22:E22"/>

</xml_diff>

<commit_message>
JEST: kapi kapatma komutu acik nokta olmaktan cikarildi
Kapatma komutu (butona basildi bilgisi) arac tarafinda yonetilmektedir;
bu fonksiyon icin yeni bir cikis kullanilmaz. Ilgili acik nokta notu
kaldirildi ve 2.a / 2.b / 2.c teknik karsiliklarina acikca yazildi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1jP1JN4GEcVEbhfkZatnJ
</commit_message>
<xml_diff>
--- a/JEST_SOFTWARE_KTP_Guncel.xlsx
+++ b/JEST_SOFTWARE_KTP_Guncel.xlsx
@@ -687,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -961,8 +961,9 @@
 2. Ekranda Telltale 1 aktif edilir.
 3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
 4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
-5. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
-6. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
+5. Süre dolduğunda kapı kapatma komutu, araç tarafında yönetilen mevcut kapı kumanda yolu üzerinden verilir; bu fonksiyon için yeni bir çıkış kullanılmaz.
+6. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+7. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -993,8 +994,9 @@
 2. Ekranda Telltale 2 aktif edilir.
 3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
 4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
-5. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
-6. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
+5. Süre dolduğunda kapı kapatma komutu, araç tarafında yönetilen mevcut kapı kumanda yolu üzerinden verilir; bu fonksiyon için yeni bir çıkış kullanılmaz.
+6. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+7. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -1025,8 +1027,9 @@
 2. Ekranda Telltale 3 aktif edilir.
 3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
 4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
-5. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
-6. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
+5. Süre dolduğunda kapı kapatma komutu, araç tarafında yönetilen mevcut kapı kumanda yolu üzerinden verilir; bu fonksiyon için yeni bir çıkış kullanılmaz.
+6. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+7. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1197,30 +1200,22 @@
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>1) I/O listesinde kapı kapatma komutuna ait bir çıkış bulunmamaktadır. Autoclose süresi dolduğunda kapının hangi çıkış üzerinden kapatılacağı (TENU B4 kapı butonu hattı veya başka bir yol) netleştirilerek bu tabloya işlenmelidir.</t>
+          <t>1) MUX C-C (16) çıkışı PWM ile sürülmektedir (TRUE = PWM 250, FALSE = PWM 0). PWM frekansı ve fotosel trigger girişinde oluşan ortalama gerilim ile dalgalanma araç üzerinde ölçülerek doğrulanmalıdır; trigger girişi seviye bekliyorsa PWM'in sürekli 12V gibi algılandığı teyit edilmelidir.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>2) MUX C-C (16) çıkışı PWM ile sürülmektedir (TRUE = PWM 250, FALSE = PWM 0). PWM frekansı ve fotosel trigger girişinde oluşan ortalama gerilim ile dalgalanma araç üzerinde ölçülerek doğrulanmalıdır; trigger girişi seviye bekliyorsa PWM'in sürekli 12V gibi algılandığı teyit edilmelidir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="42" customHeight="1">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>3) Fotosel çıkış seviyesi 12V'tur. MUX C-A (12) girişinin bu seviyeyi dijital giriş olarak doğru okuduğu araç üzerinde doğrulanmalıdır.</t>
+          <t>2) Fotosel çıkış seviyesi 12V'tur. MUX C-A (12) girişinin bu seviyeyi dijital giriş olarak doğru okuduğu araç üzerinde doğrulanmalıdır.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A22:E22"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="A22:E22"/>
     <mergeCell ref="A18:E18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
JEST: gecis kosulu tam acik svici olarak netlestirildi
Fotosel algilama alani gecisi kapi butonuna degil, TENU A5 on kanat tam
acik svicinin durumuna baglidir. 1.a metni ve KTP MADDE 3-4 bu dile
cevrildi; role kontaginin sasaye kapanmasi ve birakinca yaklasik 12V
okunmasi kabul kriterine eklendi.

Role pin detayi SOFTWARE teknik karsiligindan cikarildi; harness
bilgisi olarak blok semada kalir.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1jP1JN4GEcVEbhfkZatnJ
</commit_message>
<xml_diff>
--- a/JEST_SOFTWARE_KTP_Guncel.xlsx
+++ b/JEST_SOFTWARE_KTP_Guncel.xlsx
@@ -777,7 +777,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Fotosel, tetikleme (IN) girişinin seviyesine göre iki farklı algılama alanında çalışır: kapı tam açık olduğu durumda trigger ucuna 12V verilir ve fotosel 12 beamlik geniş alanda çalışır. Kapı tam açık sinyali araç tarafında hâli hazırda bulunmadığından, TENU üzerindeki ön kanat tam açık sinyalinden bir röle bağlantısı kurulur ve rölenin çıkışı araç yazılımına kapı full açık sinyali olarak verilir. Kapı full açık olduğu durumda araç yazılımı fotoselin trigger ucuna 12V gönderir; kapı tam açık konumundan çıktığı anda 12V kesilir ve 0V verilir. 12V kesildiği anda fotosel 12 beamden 2 beame düşer. Böylece kapı ağzına giren kanatlar algılama alanını tetiklemez, kapı ağzının ortasında duran yolcu ise görülmeye devam eder.</t>
+          <t>Fotosel, tetikleme (IN) girişinin seviyesine göre iki farklı algılama alanında çalışır: kapı tam açık olduğu durumda trigger ucuna 12V verilir ve fotosel 12 beamlik geniş alanda çalışır. Kapı tam açık sinyali araç tarafında hâli hazırda bulunmadığından, TENU üzerindeki A5 ön kanat tam açık sinyalinden bir röle bağlantısı kurulur ve rölenin çıkışı araç yazılımına kapı full açık sinyali olarak verilir. Kapı, tam açık sviçini geçtiği sürece full açık kabul edilir. Kapı full açık olduğu durumda araç yazılımı fotoselin trigger ucuna 12V gönderir; kapı tam açık konumundan çıkıp sviç bıraktığı anda 12V kesilir ve 0V verilir. 12V kesildiği anda fotosel 12 beamden 2 beame düşer. Böylece kapı ağzına giren kanatlar algılama alanını tetiklemez, kapı ağzının ortasında duran yolcu ise görülmeye devam eder. Alan geçişi kapı butonuna basılmasına değil, tam açık sviçinin durumuna bağlıdır.</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -785,9 +785,9 @@
           <t>1. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
 2. MUX C-C (16) — Analog (PWM) çıkış. TRUE durumunda PWM 250 sürülür ve fotosel trigger ucunda 12V oluşur; FALSE durumunda PWM 0 sürülür ve trigger ucu 0V olur.
 3. MUX B-A (31) &lt; 0,5V (kapı full açık) → MUX C-C (16) TRUE, PWM 250, trigger ucunda 12V → 12 beam (geniş algılama alanı).
-4. MUX B-A (31) &gt; 0,5V (kapı full açık değil) → MUX C-C (16) FALSE, PWM 0, trigger ucu 0V → 2 beam (dar algılama alanı).
+4. Kapı tam açık sviçi bıraktığında MUX B-A (31) &gt; 0,5V (kapı full açık değil) → MUX C-C (16) FALSE, PWM 0, trigger ucu 0V → 2 beam (dar algılama alanı).
 5. Kapı kapalı konumdayken ve kapı açılırken çıkış FALSE tutulur; kapı tam açık konuma ulaştığında yeniden TRUE yapılır.
-6. Röle bobini TENU ön kanat tam açık çıkışına bağlanır; röle kontağının çıkışı MUX B-A (31) girişine verilir.</t>
+6. Geçiş koşulu kapı butonu değil, kapı tam açık sinyalinin durumudur.</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -1512,7 +1512,7 @@
       <c r="C11" s="11" t="n"/>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>Kapı tam açıkken röle çekmeli ve MUX B-A (31) girişinde 0,5V ALTI (&lt; 500 mV) değer okunmalıdır. Araç yazılımı MUX C-C (16) çıkışını TRUE yaparak PWM 250 sürmeli, fotosel trigger ucunda 12V ölçülmelidir. Fotosel 12 beam (geniş algılama alanı) modunda olmalıdır. Ölçülen değerler bu forma kaydedilmelidir.</t>
+          <t>Kapı tam açık sviçini geçtiğinde röle çekmeli, kontak şaseye kapanmalı ve MUX B-A (31) girişinde 0,5V ALTI (&lt; 500 mV) değer okunmalıdır. Araç yazılımı MUX C-C (16) çıkışını TRUE yaparak PWM 250 sürmeli, fotosel trigger ucunda 12V ölçülmelidir. Fotosel 12 beam (geniş algılama alanı) modunda olmalıdır. Ölçülen değerler bu forma kaydedilmelidir.</t>
         </is>
       </c>
       <c r="E11" s="11" t="n"/>
@@ -1586,7 +1586,7 @@
       <c r="C14" s="18" t="n"/>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Kapı tam açık konumdan çıkarılır (kapanmaya başlatılır). MUX B-A (31) girişi, MUX C-C (16) çıkışı ve fotosel trigger ucu eş zamanlı kaydedilir.</t>
+          <t>Kapı tam açık konumdan çıkarılır (kapanmaya başlatılır). TENU A5 tam açık sviçi, MUX B-A (31) girişi, MUX C-C (16) çıkışı ve fotosel trigger ucu eş zamanlı kaydedilir.</t>
         </is>
       </c>
       <c r="E14" s="18" t="n"/>
@@ -1612,7 +1612,7 @@
       <c r="C15" s="11" t="n"/>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>Kapı tam açık konumdan çıktığı anda MUX B-A (31) girişinde 0,5V ÜSTÜ değer okunmalı, MUX C-C (16) çıkışı FALSE olmalı (PWM 0) ve trigger ucu 0V'a düşmelidir. Fotosel 2 beam (dar algılama alanı) moduna geçmelidir. Geçiş, kanatların ışın alanına girmesinden ÖNCE tamamlanmalıdır.</t>
+          <t>Kapı tam açık sviçini bıraktığı anda röle bırakmalı ve MUX B-A (31) girişinde 0,5V ÜSTÜ (yaklaşık 12V) değer okunmalı, MUX C-C (16) çıkışı FALSE olmalı (PWM 0) ve trigger ucu 0V'a düşmelidir. Fotosel 2 beam (dar algılama alanı) moduna geçmelidir. Geçiş, kanatların ışın alanına girmesinden ÖNCE tamamlanmalıdır.</t>
         </is>
       </c>
       <c r="E15" s="11" t="n"/>

</xml_diff>

<commit_message>
JEST: SOFTWARE'den I/O tipleri cikarildi, KTP 14 maddeye genisletildi
SOFTWARE teknik karsiliklarinda 'Analog giris / Dijital cikis' ibareleri
kaldirildi; tip bilgisi HARNESS I/O tablosunda kalir, gereksinimde yalnizca
pin ve seviye yazilidir.

KTP ilk bes maddesi pin bazinda seviye kontrolu olacak sekilde yeniden
kurgulandi: C-A (11), C-A (12), B-A (31), C-C (16) ve C-B (1) pinlerinin
her biri iki durumda da olculup forma kaydedilir. Kalan dokuz madde
fonksiyonel testleri kapsar. Madde metinleri kisaltildi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1jP1JN4GEcVEbhfkZatnJ
</commit_message>
<xml_diff>
--- a/JEST_SOFTWARE_KTP_Guncel.xlsx
+++ b/JEST_SOFTWARE_KTP_Guncel.xlsx
@@ -753,7 +753,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>1. MUX C-A (11) — Analog giriş. 8V üstü okunduğunda fotosel/autoclose butonu BASILI (fonksiyon aktif); 8V altı okunduğunda BIRAKILMIŞ (fonksiyon deaktif).
+          <t>1. MUX C-A (11) — 8V üstü okunduğunda fotosel/autoclose butonu BASILI (fonksiyon aktif); 8V altı okunduğunda BIRAKILMIŞ (fonksiyon deaktif).
 2. Giriş 8V üstü okunduğunda fotosel fonksiyonu devrededir ve autoclose fonksiyonunun iki koşulundan biri sağlanmış olur.
 3. Giriş 8V altı okunduğunda MUX engel değerlendirmesi yapmaz ve autoclose aktif olmaz.</t>
         </is>
@@ -782,8 +782,8 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>1. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
-2. MUX C-C (16) — Analog (PWM) çıkış. TRUE durumunda PWM 250 sürülür ve fotosel trigger ucunda 12V oluşur; FALSE durumunda PWM 0 sürülür ve trigger ucu 0V olur.
+          <t>1. MUX B-A (31) — 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+2. MUX C-C (16) — TRUE durumunda PWM 250 sürülür ve fotosel trigger ucunda 12V oluşur; FALSE durumunda PWM 0 sürülür ve trigger ucu 0V olur.
 3. MUX B-A (31) &lt; 0,5V (kapı full açık) → MUX C-C (16) TRUE, PWM 250, trigger ucunda 12V → 12 beam (geniş algılama alanı).
 4. Kapı tam açık sviçi bıraktığında MUX B-A (31) &gt; 0,5V (kapı full açık değil) → MUX C-C (16) FALSE, PWM 0, trigger ucu 0V → 2 beam (dar algılama alanı).
 5. Kapı kapalı konumdayken ve kapı açılırken çıkış FALSE tutulur; kapı tam açık konuma ulaştığında yeniden TRUE yapılır.
@@ -814,9 +814,9 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>1. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.
+          <t>1. MUX C-A (12) — 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.
 2. MUX C-A (12) &gt; 8V (engel var) → MUX C-B (1) TRUE yapılır.
-3. MUX C-B (1) — Dijital çıkış. TRUE gönderildiğinde TENU C3'e kapı sıkışma bilgisi iletilir; FALSE'ta hat serbest bırakılır.
+3. MUX C-B (1) — TRUE gönderildiğinde TENU C3'e kapı sıkışma bilgisi iletilir; FALSE'ta hat serbest bırakılır.
 4. Bu bilgi TENU C3 (kapı sıkışma / emniyet fitili) girişine gönderilir; ünite kapıyı durdurur ve geri açar.</t>
         </is>
       </c>
@@ -874,7 +874,7 @@
       <c r="D7" s="5" t="inlineStr">
         <is>
           <t>1. Cluster autoclose seçimi (deaktif dahil) fotosel fonksiyonunu etkilemez.
-2. Koşul yalnızca buton hattının 8V üstü okunmasıdır: MUX C-A (11) — Analog giriş. 8V üstü okunduğunda fotosel/autoclose butonu BASILI (fonksiyon aktif); 8V altı okunduğunda BIRAKILMIŞ (fonksiyon deaktif).</t>
+2. Koşul yalnızca buton hattının 8V üstü okunmasıdır: MUX C-A (11) — 8V üstü okunduğunda fotosel/autoclose butonu BASILI (fonksiyon aktif); 8V altı okunduğunda BIRAKILMIŞ (fonksiyon deaktif).</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -930,7 +930,7 @@
       <c r="D9" s="5" t="inlineStr">
         <is>
           <t>1. Cluster → araç yazılımına CAN mesajı (seçilen autoclose süresi) — seçilen süre 3 / 10 / 14 olmalıdır (0 = deaktif).
-2. MUX C-A (11) — Analog giriş. 8V üstü okunduğunda fotosel/autoclose butonu BASILI (fonksiyon aktif); 8V altı okunduğunda BIRAKILMIŞ (fonksiyon deaktif). — 8V üstü okunmalıdır.</t>
+2. MUX C-A (11) — 8V üstü okunduğunda fotosel/autoclose butonu BASILI (fonksiyon aktif); 8V altı okunduğunda BIRAKILMIŞ (fonksiyon deaktif). — 8V üstü okunmalıdır.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -962,8 +962,8 @@
 3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
 4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
 5. Süre dolduğunda kapı kapatma komutu, araç tarafında yönetilen mevcut kapı kumanda yolu üzerinden verilir; bu fonksiyon için yeni bir çıkış kullanılmaz.
-6. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
-7. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
+6. MUX B-A (31) — 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+7. MUX C-A (12) — 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -995,8 +995,8 @@
 3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
 4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
 5. Süre dolduğunda kapı kapatma komutu, araç tarafında yönetilen mevcut kapı kumanda yolu üzerinden verilir; bu fonksiyon için yeni bir çıkış kullanılmaz.
-6. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
-7. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
+6. MUX B-A (31) — 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+7. MUX C-A (12) — 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -1028,8 +1028,8 @@
 3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
 4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
 5. Süre dolduğunda kapı kapatma komutu, araç tarafında yönetilen mevcut kapı kumanda yolu üzerinden verilir; bu fonksiyon için yeni bir çıkış kullanılmaz.
-6. MUX B-A (31) — Analog giriş. 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
-7. MUX C-A (12) — Analog giriş. 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
+6. MUX B-A (31) — 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
+7. MUX C-A (12) — 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1207,7 +1207,7 @@
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>2) Fotosel çıkış seviyesi 12V'tur. MUX C-A (12) girişinin bu seviyeyi dijital giriş olarak doğru okuduğu araç üzerinde doğrulanmalıdır.</t>
+          <t>2) Fotosel çıkış seviyesi 12V'tur. MUX C-A (12) girişinin bu seviyeyi doğru okuduğu araç üzerinde doğrulanmalıdır.</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P49"/>
+  <dimension ref="A1:P57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1286,7 +1286,7 @@
       <c r="C2" s="18" t="n"/>
       <c r="D2" s="19" t="inlineStr">
         <is>
-          <t>Fotosel/autoclose butonu basılı konuma getirilir ve MUX C-A (11) analog girişi ölçülür. Ardından buton bırakılır ve ölçüm tekrarlanır. Her iki konumda fotoselin besleme hattı da kontrol edilir.</t>
+          <t>Buton basılı ve bırakılmış konumlarda MUX C-A (11) girişi ile fotosel B+ besleme hattı ölçülür.</t>
         </is>
       </c>
       <c r="E2" s="18" t="n"/>
@@ -1312,7 +1312,7 @@
       <c r="C3" s="11" t="n"/>
       <c r="D3" s="23" t="inlineStr">
         <is>
-          <t>Buton basılıyken MUX C-A (11) girişinde 8V ÜSTÜ değer okunmalı ve fotosel beslemede olmalıdır. Buton bırakıldığında 8V ALTI değer okunmalı ve fotosel beslemesiz kalmalıdır. Okunan gerilim değerleri bu forma kaydedilmelidir.</t>
+          <t>Basılıyken C-A (11) girişinde 8V ÜSTÜ okunmalı ve fotosel beslemede olmalıdır. Bırakıldığında 8V ALTI okunmalı, besleme kesilmelidir. Ölçülen değerler forma kaydedilir.</t>
         </is>
       </c>
       <c r="E3" s="11" t="n"/>
@@ -1386,7 +1386,7 @@
       <c r="C6" s="18" t="n"/>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Buton basılı konumdayken fotosel enerjilendirilir; gösterge LED'leri ve ilk enerjilenme davranışı gözlenir. Fotosel önüne engel konulup kaldırılarak MUX C-A (12) analog girişi izlenir.</t>
+          <t>Fotosel önüne engel konup kaldırılarak MUX C-A (12) girişi ölçülür.</t>
         </is>
       </c>
       <c r="E6" s="18" t="n"/>
@@ -1412,7 +1412,7 @@
       <c r="C7" s="11" t="n"/>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>Engel konulduğunda MUX C-A (12) girişinde 8V ÜSTÜ değer okunmalı, engel kaldırıldığında 8V ALTI değere dönmelidir. Okunan gerilim değerleri bu forma kaydedilmelidir.</t>
+          <t>Engel varken 8V ÜSTÜ, engel yokken 8V ALTI okunmalıdır. Ölçülen değerler forma kaydedilir.</t>
         </is>
       </c>
       <c r="E7" s="11" t="n"/>
@@ -1486,7 +1486,7 @@
       <c r="C10" s="18" t="n"/>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Kapı tam açık konuma getirilir. TENU ön kanat tam açık çıkışı, röle kontağı, MUX B-A (31) analog girişi, MUX C-C (16) çıkışı ve fotosel trigger ucu birlikte ölçülür.</t>
+          <t>Kapı tam açık konumda ve tam açık konumdan çıkmış durumda MUX B-A (31) girişi ölçülür.</t>
         </is>
       </c>
       <c r="E10" s="18" t="n"/>
@@ -1512,7 +1512,7 @@
       <c r="C11" s="11" t="n"/>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>Kapı tam açık sviçini geçtiğinde röle çekmeli, kontak şaseye kapanmalı ve MUX B-A (31) girişinde 0,5V ALTI (&lt; 500 mV) değer okunmalıdır. Araç yazılımı MUX C-C (16) çıkışını TRUE yaparak PWM 250 sürmeli, fotosel trigger ucunda 12V ölçülmelidir. Fotosel 12 beam (geniş algılama alanı) modunda olmalıdır. Ölçülen değerler bu forma kaydedilmelidir.</t>
+          <t>Tam açıkken (röle çekili) 0,5V ALTI, tam açık değilken (röle bırakmış) 0,5V ÜSTÜ ve yaklaşık 12V okunmalıdır. Ölçülen değerler forma kaydedilir.</t>
         </is>
       </c>
       <c r="E11" s="11" t="n"/>
@@ -1586,7 +1586,7 @@
       <c r="C14" s="18" t="n"/>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Kapı tam açık konumdan çıkarılır (kapanmaya başlatılır). TENU A5 tam açık sviçi, MUX B-A (31) girişi, MUX C-C (16) çıkışı ve fotosel trigger ucu eş zamanlı kaydedilir.</t>
+          <t>Kapı tam açıkken ve tam açık konumdan çıktıktan sonra MUX C-C (16) çıkışı ile fotosel trigger ucu osiloskopla ölçülür.</t>
         </is>
       </c>
       <c r="E14" s="18" t="n"/>
@@ -1612,7 +1612,7 @@
       <c r="C15" s="11" t="n"/>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>Kapı tam açık sviçini bıraktığı anda röle bırakmalı ve MUX B-A (31) girişinde 0,5V ÜSTÜ (yaklaşık 12V) değer okunmalı, MUX C-C (16) çıkışı FALSE olmalı (PWM 0) ve trigger ucu 0V'a düşmelidir. Fotosel 2 beam (dar algılama alanı) moduna geçmelidir. Geçiş, kanatların ışın alanına girmesinden ÖNCE tamamlanmalıdır.</t>
+          <t>Tam açıkken çıkış TRUE (PWM 250), trigger ucunda 12V olmalıdır. Tam açık konumdan çıkınca çıkış FALSE (PWM 0), trigger ucu 0V'a düşmelidir. Trigger ucundaki ortalama gerilim ve dalgalanma kaydedilir.</t>
         </is>
       </c>
       <c r="E15" s="11" t="n"/>
@@ -1686,7 +1686,7 @@
       <c r="C18" s="18" t="n"/>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Fotosel önünde engel bulunmadan kapı tam açıktan tam kapalıya kadar kapatılır. MUX C-A (12) girişi kapanma boyunca kaydedilir.</t>
+          <t>Fotosel önüne engel konup kaldırılarak MUX C-B (1) çıkışı ve TENU C3 hattı ölçülür.</t>
         </is>
       </c>
       <c r="E18" s="18" t="n"/>
@@ -1712,7 +1712,7 @@
       <c r="C19" s="11" t="n"/>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t>Kapanma boyunca MUX C-A (12) girişi 8V ALTINDA kalmalı; kapı kanatları fotoseli tetiklememelidir. Kapı durdurulmadan, kesintisiz olarak tam kapalı konuma ulaşmalıdır.</t>
+          <t>Engel varken çıkış TRUE ve TENU C3 hattında kapı sıkışma bilgisi görülmelidir. Engel yokken çıkış FALSE ve hat serbest olmalıdır.</t>
         </is>
       </c>
       <c r="E19" s="11" t="n"/>
@@ -1786,7 +1786,7 @@
       <c r="C22" s="18" t="n"/>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Kapı açıkken fotosel önüne engel konur ve kapatma isteği gönderilir. MUX C-A (12) girişi, MUX C-B (1) çıkışı, TENU C3 hattı ve kapı hareketi izlenir.</t>
+          <t>Kapı kapalıdan tam açığa, oradan tekrar kapalıya götürülür. Röle kontağı, MUX B-A (31), MUX C-C (16) ve trigger ucu eş zamanlı kaydedilir.</t>
         </is>
       </c>
       <c r="E22" s="18" t="n"/>
@@ -1812,7 +1812,7 @@
       <c r="C23" s="11" t="n"/>
       <c r="D23" s="23" t="inlineStr">
         <is>
-          <t>MUX C-A (12) girişinde 8V ÜSTÜ değer okunmalı, MUX C-B (1) çıkışı TRUE olmalı ve TENU C3 hattına kapı sıkışma bilgisi iletilmelidir. Kapı kapanmamalı; kapanmakta ise durdurulup geri açılmalıdır. Komut şoför butonundan, dış butondan veya uzaktan kumandadan gelse dahi kapı kapanmamalıdır.</t>
+          <t>Tam açık sviçi çekince röle çeker, B-A (31) 0,5V altına iner, trigger 12V olur ve fotosel 12 beam moduna geçer. Sviç bırakınca trigger 0V olur ve 2 beam moduna geçer. Geçiş, kanatlar ışın alanına girmeden önce tamamlanmalıdır.</t>
         </is>
       </c>
       <c r="E23" s="11" t="n"/>
@@ -1886,7 +1886,7 @@
       <c r="C26" s="18" t="n"/>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>Engel kaldırılır. MUX C-A (12) girişi, MUX C-B (1) çıkışı ve TENU C3 hattı izlenir. Ardından gerçek emniyet fitiline elle basılarak kapı kontrol ünitesinin tepkisi kontrol edilir.</t>
+          <t>Fotosel önünde engel bulunmadan kapı tam açıktan tam kapalıya kapatılır; MUX C-A (12) kaydedilir.</t>
         </is>
       </c>
       <c r="E26" s="18" t="n"/>
@@ -1912,7 +1912,7 @@
       <c r="C27" s="11" t="n"/>
       <c r="D27" s="23" t="inlineStr">
         <is>
-          <t>Engel kalktığında MUX C-A (12) 8V ALTINA inmeli, MUX C-B (1) çıkışı FALSE olmalı ve TENU C3 hattı serbest bırakılmalıdır; kapatma isteği tekrar kabul edilmelidir. Çıkış FALSE iken hat üzerinde yük oluşturmamalı, gerçek emniyet fitilinin çalışması etkilenmemelidir.</t>
+          <t>Kapanma boyunca C-A (12) 8V altında kalmalı, kapı kanatları fotoseli tetiklememelidir. Kapı durdurulmadan tam kapalı konuma ulaşmalıdır.</t>
         </is>
       </c>
       <c r="E27" s="11" t="n"/>
@@ -1986,7 +1986,7 @@
       <c r="C30" s="18" t="n"/>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>Cluster üzerinden sırasıyla 10 sn, 14 sn ve 3 sn seçilir. Her seçimde buton basılı, kapı tam açık konuma getirilerek engelsiz beklenir ve kapanma süresi kronometre ile ölçülür.</t>
+          <t>Kapı açıkken fotosel önüne engel konur; şoför butonundan, dış butondan ve uzaktan kumandadan kapatma isteği gönderilir. Ardından engel kaldırılıp kapatma tekrarlanır.</t>
         </is>
       </c>
       <c r="E30" s="18" t="n"/>
@@ -2012,7 +2012,7 @@
       <c r="C31" s="11" t="n"/>
       <c r="D31" s="23" t="inlineStr">
         <is>
-          <t>Her seçimde ekranda ilgili telltale görüntülenmelidir (10 sn → Telltale 1, 14 sn → Telltale 2, 3 sn → Telltale 3). Geri sayım, MUX B-A (31) girişi 0,5V altına indiği anda başlamalı ve kapı seçili süre sonunda kapanmalıdır. Ölçülen süreler bu forma kaydedilmelidir.</t>
+          <t>Engel varken hiçbir komutla kapı kapanmamalı, kapanmakta ise durdurulup geri açılmalıdır. Engel kalktığında C-B (1) FALSE olmalı ve kapı kapanabilmelidir.</t>
         </is>
       </c>
       <c r="E31" s="11" t="n"/>
@@ -2086,7 +2086,7 @@
       <c r="C34" s="18" t="n"/>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>Auto Close 10 sn seçiliyken sayaç çalışırken fotosel önüne engel konur, bir süre bekletilip kaldırılır.</t>
+          <t>Gerçek emniyet fitiline elle basılarak kapı kontrol ünitesinin tepkisi gözlenir.</t>
         </is>
       </c>
       <c r="E34" s="18" t="n"/>
@@ -2112,7 +2112,7 @@
       <c r="C35" s="11" t="n"/>
       <c r="D35" s="23" t="inlineStr">
         <is>
-          <t>MUX C-A (12) 8V üstüne çıktığında sayaç sıfırlanmalıdır. Kapı ancak engel kalktıktan sonra kesintisiz 10 saniye geçince kapanmalıdır.</t>
+          <t>Kapı kontrol ünitesi normal tepkisini vermelidir; MUX'un TENU C3 hattına bağlı olması emniyet fitilinin çalışmasını etkilememelidir.</t>
         </is>
       </c>
       <c r="E35" s="11" t="n"/>
@@ -2186,7 +2186,7 @@
       <c r="C38" s="18" t="n"/>
       <c r="D38" s="19" t="inlineStr">
         <is>
-          <t>Cluster üzerinden autoclose deaktif seçilir; kapı tam açık konuma getirilip 20 saniyeden uzun süre beklenir. Ardından buton bırakılmış durumda 10 sn seçilerek aynı bekleme tekrarlanır.</t>
+          <t>Cluster 10 sn + buton basılı, cluster 10 sn + buton bırakılmış, cluster deaktif + buton basılı kombinasyonları denenir; her birinde kapı tam açıkken 20 saniyeden uzun beklenir.</t>
         </is>
       </c>
       <c r="E38" s="18" t="n"/>
@@ -2212,7 +2212,7 @@
       <c r="C39" s="11" t="n"/>
       <c r="D39" s="23" t="inlineStr">
         <is>
-          <t>Her iki durumda da ekranda autoclose telltale'i görüntülenmemeli ve kapı kendiliğinden kapanmamalıdır. Fotosel fonksiyonu (engel algılandığında kapının kapanmaması) çalışmaya devam etmelidir.</t>
+          <t>Yalnızca süre seçili VE buton basılı kombinasyonunda kapı otomatik kapanmalıdır. Diğerlerinde kapı kapanmamalı, telltale görüntülenmemelidir.</t>
         </is>
       </c>
       <c r="E39" s="11" t="n"/>
@@ -2286,7 +2286,7 @@
       <c r="C42" s="18" t="n"/>
       <c r="D42" s="19" t="inlineStr">
         <is>
-          <t>Sayaç çalışırken sırasıyla acil durum, yangın algılama (MUX E (A) 18 GND / MUX E (A) 17 12V) ve blokaj butonu (MUX C (A) 16 / MUX C (A) 23) aktif edilir; her biri ayrı ayrı denenip kaldırılır.</t>
+          <t>Cluster üzerinden sırasıyla 10 sn, 14 sn ve 3 sn seçilir; her seçimde kapı tam açıkken engelsiz beklenir ve süre kronometre ile ölçülür.</t>
         </is>
       </c>
       <c r="E42" s="18" t="n"/>
@@ -2312,7 +2312,7 @@
       <c r="C43" s="11" t="n"/>
       <c r="D43" s="23" t="inlineStr">
         <is>
-          <t>Her üç durumda da sayaç durmalı ve kapı kapatma komutu verilmemelidir. Durum kalktığında sayaç yeniden başlamalı ve kapı seçili süre sonunda kapanmalıdır.</t>
+          <t>İlgili telltale görüntülenmelidir (10 sn → 1, 14 sn → 2, 3 sn → 3). Geri sayım B-A (31) 0,5V altına indiğinde başlamalı, kapı seçili süre sonunda kapanmalıdır. Ölçülen süreler forma kaydedilir.</t>
         </is>
       </c>
       <c r="E43" s="11" t="n"/>
@@ -2386,7 +2386,7 @@
       <c r="C46" s="18" t="n"/>
       <c r="D46" s="19" t="inlineStr">
         <is>
-          <t>Fotosel sinyal hattı (MUX C-A 12) sökülerek geçersiz duruma getirilir, ardından geri bağlanır. Aynı işlem MUX B-A (31) full açık sinyal hattı için tekrarlanır.</t>
+          <t>Auto Close 10 sn seçiliyken sayaç çalışırken fotosel önüne engel konur, bekletilip kaldırılır; işlem sayacın başında ve sonuna yakın tekrarlanır.</t>
         </is>
       </c>
       <c r="E46" s="18" t="n"/>
@@ -2412,7 +2412,7 @@
       <c r="C47" s="11" t="n"/>
       <c r="D47" s="23" t="inlineStr">
         <is>
-          <t>Araç yazılımı geçersiz seviyeyi tespit etmeli ve kapı kapatma komutu vermemelidir. Hatlar geri bağlandığında fonksiyon normal çalışmasına dönmelidir.</t>
+          <t>C-A (12) 8V üstüne çıktığı anda sayaç sıfırlanmalıdır. Kapı ancak engel kalktıktan sonra kesintisiz 10 saniye geçince kapanmalıdır.</t>
         </is>
       </c>
       <c r="E47" s="11" t="n"/>
@@ -2472,14 +2472,216 @@
       <c r="O49" s="27" t="n"/>
       <c r="P49" s="29" t="n"/>
     </row>
+    <row r="50" ht="32" customHeight="1">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>MADDE 13 :</t>
+        </is>
+      </c>
+      <c r="B50" s="17" t="inlineStr">
+        <is>
+          <t>PROSEDÜR</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="n"/>
+      <c r="D50" s="19" t="inlineStr">
+        <is>
+          <t>Sayaç çalışırken sırasıyla acil durum, yangın algılama (MUX E (A) 18 / E (A) 17) ve blokaj butonu (MUX C (A) 16 / C (A) 23) aktif edilip kaldırılır.</t>
+        </is>
+      </c>
+      <c r="E50" s="18" t="n"/>
+      <c r="F50" s="18" t="n"/>
+      <c r="G50" s="18" t="n"/>
+      <c r="H50" s="18" t="n"/>
+      <c r="I50" s="18" t="n"/>
+      <c r="J50" s="18" t="n"/>
+      <c r="K50" s="18" t="n"/>
+      <c r="L50" s="18" t="n"/>
+      <c r="M50" s="18" t="n"/>
+      <c r="N50" s="18" t="n"/>
+      <c r="O50" s="18" t="n"/>
+      <c r="P50" s="20" t="n"/>
+    </row>
+    <row r="51" ht="36" customHeight="1">
+      <c r="A51" s="21" t="n"/>
+      <c r="B51" s="22" t="inlineStr">
+        <is>
+          <t>KABUL KRİTERİ</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="n"/>
+      <c r="D51" s="23" t="inlineStr">
+        <is>
+          <t>Her üç durumda da sayaç durmalı ve kapatma komutu verilmemelidir. İlgili girişlerde okunan seviyeler forma kaydedilir. Durum kalkınca sayaç yeniden başlamalıdır.</t>
+        </is>
+      </c>
+      <c r="E51" s="11" t="n"/>
+      <c r="F51" s="11" t="n"/>
+      <c r="G51" s="11" t="n"/>
+      <c r="H51" s="11" t="n"/>
+      <c r="I51" s="11" t="n"/>
+      <c r="J51" s="11" t="n"/>
+      <c r="K51" s="11" t="n"/>
+      <c r="L51" s="11" t="n"/>
+      <c r="M51" s="11" t="n"/>
+      <c r="N51" s="11" t="n"/>
+      <c r="O51" s="11" t="n"/>
+      <c r="P51" s="24" t="n"/>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="21" t="n"/>
+      <c r="B52" s="22" t="inlineStr">
+        <is>
+          <t>SONUÇ</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="n"/>
+      <c r="D52" s="23" t="inlineStr"/>
+      <c r="E52" s="11" t="n"/>
+      <c r="F52" s="11" t="n"/>
+      <c r="G52" s="11" t="n"/>
+      <c r="H52" s="11" t="n"/>
+      <c r="I52" s="11" t="n"/>
+      <c r="J52" s="11" t="n"/>
+      <c r="K52" s="11" t="n"/>
+      <c r="L52" s="11" t="n"/>
+      <c r="M52" s="11" t="n"/>
+      <c r="N52" s="11" t="n"/>
+      <c r="O52" s="11" t="n"/>
+      <c r="P52" s="24" t="n"/>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="25" t="n"/>
+      <c r="B53" s="26" t="inlineStr">
+        <is>
+          <t>OK / NOK</t>
+        </is>
+      </c>
+      <c r="C53" s="27" t="n"/>
+      <c r="D53" s="28" t="inlineStr"/>
+      <c r="E53" s="27" t="n"/>
+      <c r="F53" s="27" t="n"/>
+      <c r="G53" s="27" t="n"/>
+      <c r="H53" s="27" t="n"/>
+      <c r="I53" s="27" t="n"/>
+      <c r="J53" s="27" t="n"/>
+      <c r="K53" s="27" t="n"/>
+      <c r="L53" s="27" t="n"/>
+      <c r="M53" s="27" t="n"/>
+      <c r="N53" s="27" t="n"/>
+      <c r="O53" s="27" t="n"/>
+      <c r="P53" s="29" t="n"/>
+    </row>
+    <row r="54" ht="32" customHeight="1">
+      <c r="A54" s="16" t="inlineStr">
+        <is>
+          <t>MADDE 14 :</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="inlineStr">
+        <is>
+          <t>PROSEDÜR</t>
+        </is>
+      </c>
+      <c r="C54" s="18" t="n"/>
+      <c r="D54" s="19" t="inlineStr">
+        <is>
+          <t>MUX C-A (12), MUX B-A (31) ve MUX C-A (11) hatları sırasıyla sökülüp geri bağlanır.</t>
+        </is>
+      </c>
+      <c r="E54" s="18" t="n"/>
+      <c r="F54" s="18" t="n"/>
+      <c r="G54" s="18" t="n"/>
+      <c r="H54" s="18" t="n"/>
+      <c r="I54" s="18" t="n"/>
+      <c r="J54" s="18" t="n"/>
+      <c r="K54" s="18" t="n"/>
+      <c r="L54" s="18" t="n"/>
+      <c r="M54" s="18" t="n"/>
+      <c r="N54" s="18" t="n"/>
+      <c r="O54" s="18" t="n"/>
+      <c r="P54" s="20" t="n"/>
+    </row>
+    <row r="55" ht="36" customHeight="1">
+      <c r="A55" s="21" t="n"/>
+      <c r="B55" s="22" t="inlineStr">
+        <is>
+          <t>KABUL KRİTERİ</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="n"/>
+      <c r="D55" s="23" t="inlineStr">
+        <is>
+          <t>Her durumda araç yazılımı geçersiz seviyeyi tespit etmeli ve kapatma komutu vermemelidir. Hat geri bağlandığında fonksiyon normal çalışmasına dönmelidir.</t>
+        </is>
+      </c>
+      <c r="E55" s="11" t="n"/>
+      <c r="F55" s="11" t="n"/>
+      <c r="G55" s="11" t="n"/>
+      <c r="H55" s="11" t="n"/>
+      <c r="I55" s="11" t="n"/>
+      <c r="J55" s="11" t="n"/>
+      <c r="K55" s="11" t="n"/>
+      <c r="L55" s="11" t="n"/>
+      <c r="M55" s="11" t="n"/>
+      <c r="N55" s="11" t="n"/>
+      <c r="O55" s="11" t="n"/>
+      <c r="P55" s="24" t="n"/>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="21" t="n"/>
+      <c r="B56" s="22" t="inlineStr">
+        <is>
+          <t>SONUÇ</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="n"/>
+      <c r="D56" s="23" t="inlineStr"/>
+      <c r="E56" s="11" t="n"/>
+      <c r="F56" s="11" t="n"/>
+      <c r="G56" s="11" t="n"/>
+      <c r="H56" s="11" t="n"/>
+      <c r="I56" s="11" t="n"/>
+      <c r="J56" s="11" t="n"/>
+      <c r="K56" s="11" t="n"/>
+      <c r="L56" s="11" t="n"/>
+      <c r="M56" s="11" t="n"/>
+      <c r="N56" s="11" t="n"/>
+      <c r="O56" s="11" t="n"/>
+      <c r="P56" s="24" t="n"/>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="25" t="n"/>
+      <c r="B57" s="26" t="inlineStr">
+        <is>
+          <t>OK / NOK</t>
+        </is>
+      </c>
+      <c r="C57" s="27" t="n"/>
+      <c r="D57" s="28" t="inlineStr"/>
+      <c r="E57" s="27" t="n"/>
+      <c r="F57" s="27" t="n"/>
+      <c r="G57" s="27" t="n"/>
+      <c r="H57" s="27" t="n"/>
+      <c r="I57" s="27" t="n"/>
+      <c r="J57" s="27" t="n"/>
+      <c r="K57" s="27" t="n"/>
+      <c r="L57" s="27" t="n"/>
+      <c r="M57" s="27" t="n"/>
+      <c r="N57" s="27" t="n"/>
+      <c r="O57" s="27" t="n"/>
+      <c r="P57" s="29" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="109">
+  <mergeCells count="127">
     <mergeCell ref="D18:P18"/>
     <mergeCell ref="D3:P3"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="A30:A33"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="D25:P25"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="D55:P55"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="D5:P5"/>
@@ -2498,8 +2700,10 @@
     <mergeCell ref="B49:C49"/>
     <mergeCell ref="A10:A13"/>
     <mergeCell ref="A22:A25"/>
+    <mergeCell ref="B55:C55"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B51:C51"/>
     <mergeCell ref="A34:A37"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="D7:P7"/>
@@ -2509,6 +2713,7 @@
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="D4:P4"/>
     <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D56:P56"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="D8:P8"/>
@@ -2516,12 +2721,15 @@
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="D33:P33"/>
     <mergeCell ref="D42:P42"/>
+    <mergeCell ref="D51:P51"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="D35:P35"/>
+    <mergeCell ref="D50:P50"/>
     <mergeCell ref="D44:P44"/>
     <mergeCell ref="D19:P19"/>
     <mergeCell ref="D34:P34"/>
+    <mergeCell ref="B53:C53"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="A46:A49"/>
     <mergeCell ref="A1:P1"/>
@@ -2533,16 +2741,21 @@
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="A38:A41"/>
     <mergeCell ref="D48:P48"/>
+    <mergeCell ref="B54:C54"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="D9:P9"/>
+    <mergeCell ref="B56:C56"/>
     <mergeCell ref="D15:P15"/>
     <mergeCell ref="D24:P24"/>
     <mergeCell ref="B43:C43"/>
     <mergeCell ref="D38:P38"/>
+    <mergeCell ref="B52:C52"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="B42:C42"/>
+    <mergeCell ref="A50:A53"/>
     <mergeCell ref="D26:P26"/>
     <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B57:C57"/>
     <mergeCell ref="D10:P10"/>
     <mergeCell ref="B44:C44"/>
     <mergeCell ref="A26:A29"/>
@@ -2551,6 +2764,7 @@
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="A42:A45"/>
     <mergeCell ref="A14:A17"/>
+    <mergeCell ref="D52:P52"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D49:P49"/>
     <mergeCell ref="D2:P2"/>
@@ -2558,6 +2772,7 @@
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B45:C45"/>
+    <mergeCell ref="D53:P53"/>
     <mergeCell ref="D47:P47"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="D28:P28"/>
@@ -2572,16 +2787,19 @@
     <mergeCell ref="D29:P29"/>
     <mergeCell ref="B48:C48"/>
     <mergeCell ref="D23:P23"/>
+    <mergeCell ref="D54:P54"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="D46:P46"/>
     <mergeCell ref="D40:P40"/>
     <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D57:P57"/>
     <mergeCell ref="D32:P32"/>
     <mergeCell ref="D27:P27"/>
     <mergeCell ref="D41:P41"/>
     <mergeCell ref="D17:P17"/>
     <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B50:C50"/>
     <mergeCell ref="D43:P43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
JEST 2.a/2.b/2.c: tekrar eden pin tanimlari kaldirildi
6. ve 7. maddeler, 3. ve 4. maddelerde zaten verilen pin ve seviye
bilgisini tekrarliyordu; tanimlar gereksinim 1 ve 1.a'da bir kez
yazildigindan kaldirildi. Kapatma komutu ifadesi 'mevcut kapi butonu
uzerinden' olarak duzeltildi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1jP1JN4GEcVEbhfkZatnJ
</commit_message>
<xml_diff>
--- a/JEST_SOFTWARE_KTP_Guncel.xlsx
+++ b/JEST_SOFTWARE_KTP_Guncel.xlsx
@@ -961,9 +961,7 @@
 2. Ekranda Telltale 1 aktif edilir.
 3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
 4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
-5. Süre dolduğunda kapı kapatma komutu, araç tarafında yönetilen mevcut kapı kumanda yolu üzerinden verilir; bu fonksiyon için yeni bir çıkış kullanılmaz.
-6. MUX B-A (31) — 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
-7. MUX C-A (12) — 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
+5. Süre dolduğunda kapı kapatma komutu, araç tarafında yönetilen mevcut kapı butonu üzerinden verilir; bu fonksiyon için yeni bir çıkış kullanılmaz.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -994,9 +992,7 @@
 2. Ekranda Telltale 2 aktif edilir.
 3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
 4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
-5. Süre dolduğunda kapı kapatma komutu, araç tarafında yönetilen mevcut kapı kumanda yolu üzerinden verilir; bu fonksiyon için yeni bir çıkış kullanılmaz.
-6. MUX B-A (31) — 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
-7. MUX C-A (12) — 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
+5. Süre dolduğunda kapı kapatma komutu, araç tarafında yönetilen mevcut kapı butonu üzerinden verilir; bu fonksiyon için yeni bir çıkış kullanılmaz.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -1027,9 +1023,7 @@
 2. Ekranda Telltale 3 aktif edilir.
 3. Sayaç başlangıcı: MUX B-A (31) &lt; 0,5V okunduğunda (kapı full açık).
 4. Sayaç reset: MUX C-A (12) &gt; 8V okunduğunda (engel algılandı).
-5. Süre dolduğunda kapı kapatma komutu, araç tarafında yönetilen mevcut kapı kumanda yolu üzerinden verilir; bu fonksiyon için yeni bir çıkış kullanılmaz.
-6. MUX B-A (31) — 0,5V (500 mV) altı okunduğunda kapı full açık; 0,5V üstü okunduğunda kapı full açık değil. Sinyal, TENU ön kanat tam açık çıkışına bağlanan rölenin çıkışından alınır.
-7. MUX C-A (12) — 8V üstü okunduğunda fotosel nesne (engel) tespit etmiştir; 8V altı okunduğunda engel yoktur.</t>
+5. Süre dolduğunda kapı kapatma komutu, araç tarafında yönetilen mevcut kapı butonu üzerinden verilir; bu fonksiyon için yeni bir çıkış kullanılmaz.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">

</xml_diff>